<commit_message>
Support for CAPEX section for fuel markets
Structure mirrors that of the financial statements.

Dynamic cell behavior to be implemented in future updates.
</commit_message>
<xml_diff>
--- a/backend/financial-statements/financial-statements-template.xlsx
+++ b/backend/financial-statements/financial-statements-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8954da175e61d5af/Escritorio/IIT/NICCP-AI/backend/financial-statements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="425" documentId="10_ncr:20000_{4F2B366B-AA2F-4F18-863E-957538EF6F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B61EF10-4CEE-4B11-94C0-E906AC5F63EE}"/>
+  <xr:revisionPtr revIDLastSave="430" documentId="10_ncr:20000_{4F2B366B-AA2F-4F18-863E-957538EF6F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0C1DD64-7654-45DF-8836-D61714ABAC80}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="E-Cooking" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1779" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1779" uniqueCount="112">
   <si>
     <t>Units</t>
   </si>
@@ -363,9 +363,6 @@
   </si>
   <si>
     <t>Total CAPEX</t>
-  </si>
-  <si>
-    <t>M MGA</t>
   </si>
   <si>
     <t>years</t>
@@ -40000,7 +39997,7 @@
         <v>4</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>108</v>
+        <v>2</v>
       </c>
       <c r="D123" s="2">
         <v>0</v>
@@ -40101,13 +40098,13 @@
     </row>
     <row r="124" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A124" s="12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B124" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>108</v>
+        <v>2</v>
       </c>
       <c r="D124" s="2">
         <v>0</v>
@@ -40208,13 +40205,13 @@
     </row>
     <row r="125" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A125" s="12" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B125" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D125" s="2">
         <v>0</v>
@@ -40315,13 +40312,13 @@
     </row>
     <row r="126" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A126" s="23" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B126" s="24" t="s">
         <v>4</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>108</v>
+        <v>2</v>
       </c>
       <c r="D126" s="2">
         <v>0</v>

</xml_diff>

<commit_message>
Dynamic formula system for financial statements (P&L, BS, CF)
Implemented a scalable and customizable system for applying formulas to dynamic cells across financial statement files.

JSON structure defines formulas for each relevant sheet (e.g., P&L, Balance Sheet, Cash Flow Statement), including step-by-step operations, operands, targets, and source labels.

Initial integration and validation completed for P&L, BS, and CF statements.

Further checks will be required as more values and sheets are incorporated.
</commit_message>
<xml_diff>
--- a/backend/financial-statements/financial-statements-template.xlsx
+++ b/backend/financial-statements/financial-statements-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8954da175e61d5af/Escritorio/IIT/NICCP-AI/backend/financial-statements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="430" documentId="10_ncr:20000_{4F2B366B-AA2F-4F18-863E-957538EF6F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0C1DD64-7654-45DF-8836-D61714ABAC80}"/>
+  <xr:revisionPtr revIDLastSave="492" documentId="10_ncr:20000_{4F2B366B-AA2F-4F18-863E-957538EF6F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD38011A-356D-4212-BBC1-C0084ABE4203}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="E-Cooking" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1779" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1779" uniqueCount="117">
   <si>
     <t>Units</t>
   </si>
@@ -87,9 +87,6 @@
   </si>
   <si>
     <t>EBITDA</t>
-  </si>
-  <si>
-    <t>EBITDA (ex-Grants)</t>
   </si>
   <si>
     <t>D&amp;A</t>
@@ -215,12 +212,6 @@
     <t xml:space="preserve">Current assets </t>
   </si>
   <si>
-    <t>Total Shareholder's Equity</t>
-  </si>
-  <si>
-    <t>Other tax liabiloties</t>
-  </si>
-  <si>
     <t>Debt repayment</t>
   </si>
   <si>
@@ -243,9 +234,6 @@
   </si>
   <si>
     <t>Cash BoP</t>
-  </si>
-  <si>
-    <t>Cas EoP</t>
   </si>
   <si>
     <t>PP&amp;E - Capex</t>
@@ -375,6 +363,33 @@
   </si>
   <si>
     <t>Total Annual Depreciation</t>
+  </si>
+  <si>
+    <t>Financial Expenses</t>
+  </si>
+  <si>
+    <t>Cash EoP</t>
+  </si>
+  <si>
+    <t>Total Shareholders' Equity</t>
+  </si>
+  <si>
+    <t>Grants liabilities</t>
+  </si>
+  <si>
+    <t>Other tax liabilities</t>
+  </si>
+  <si>
+    <t>- EBITDA (ex-Grants)</t>
+  </si>
+  <si>
+    <t>CAPEX</t>
+  </si>
+  <si>
+    <t>+/- Capital increase/reduction</t>
+  </si>
+  <si>
+    <t>- Cash movement</t>
   </si>
 </sst>
 </file>
@@ -1015,7 +1030,7 @@
   <sheetData>
     <row r="1" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>5</v>
@@ -3262,7 +3277,7 @@
     </row>
     <row r="22" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>4</v>
@@ -3369,10 +3384,10 @@
     </row>
     <row r="23" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>7</v>
+        <v>15</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>8</v>
@@ -3476,7 +3491,7 @@
     </row>
     <row r="24" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>11</v>
@@ -3583,7 +3598,7 @@
     </row>
     <row r="25" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A25" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>4</v>
@@ -3690,7 +3705,7 @@
     </row>
     <row r="26" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>11</v>
@@ -3797,7 +3812,7 @@
     </row>
     <row r="27" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B27" s="10" t="s">
         <v>4</v>
@@ -3904,7 +3919,7 @@
     </row>
     <row r="28" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="4" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>11</v>
@@ -4011,7 +4026,7 @@
     </row>
     <row r="29" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="4" t="s">
-        <v>19</v>
+        <v>108</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>4</v>
@@ -4118,7 +4133,7 @@
     </row>
     <row r="30" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B30" s="10" t="s">
         <v>4</v>
@@ -4225,7 +4240,7 @@
     </row>
     <row r="31" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>4</v>
@@ -4332,10 +4347,10 @@
     </row>
     <row r="32" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A32" s="4" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>8</v>
@@ -4439,7 +4454,7 @@
     </row>
     <row r="33" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A33" s="16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>4</v>
@@ -4546,7 +4561,7 @@
     </row>
     <row r="34" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="16" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>4</v>
@@ -4653,7 +4668,7 @@
     </row>
     <row r="35" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A35" s="14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B35" s="10" t="s">
         <v>4</v>
@@ -4760,7 +4775,7 @@
     </row>
     <row r="36" spans="1:35" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A36" s="17" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="B36" s="18" t="s">
         <v>11</v>
@@ -4867,7 +4882,7 @@
     </row>
     <row r="37" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="7" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B37" s="8" t="s">
         <v>5</v>
@@ -4974,7 +4989,7 @@
     </row>
     <row r="38" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A38" s="29" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B38" s="30" t="s">
         <v>4</v>
@@ -5081,7 +5096,7 @@
     </row>
     <row r="39" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A39" s="22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>4</v>
@@ -5188,7 +5203,7 @@
     </row>
     <row r="40" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A40" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>4</v>
@@ -5295,7 +5310,7 @@
     </row>
     <row r="41" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A41" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>4</v>
@@ -5402,7 +5417,7 @@
     </row>
     <row r="42" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="29" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B42" s="30" t="s">
         <v>4</v>
@@ -5509,7 +5524,7 @@
     </row>
     <row r="43" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A43" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>4</v>
@@ -5616,7 +5631,7 @@
     </row>
     <row r="44" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A44" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>4</v>
@@ -5723,7 +5738,7 @@
     </row>
     <row r="45" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A45" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B45" s="4" t="s">
         <v>4</v>
@@ -5830,7 +5845,7 @@
     </row>
     <row r="46" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A46" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B46" s="4" t="s">
         <v>4</v>
@@ -5937,7 +5952,7 @@
     </row>
     <row r="47" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A47" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>4</v>
@@ -6044,7 +6059,7 @@
     </row>
     <row r="48" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A48" s="23" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B48" s="24" t="s">
         <v>4</v>
@@ -6151,7 +6166,7 @@
     </row>
     <row r="49" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A49" s="29" t="s">
-        <v>58</v>
+        <v>110</v>
       </c>
       <c r="B49" s="30" t="s">
         <v>4</v>
@@ -6258,7 +6273,7 @@
     </row>
     <row r="50" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A50" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>4</v>
@@ -6365,7 +6380,7 @@
     </row>
     <row r="51" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A51" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>4</v>
@@ -6472,7 +6487,7 @@
     </row>
     <row r="52" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A52" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>4</v>
@@ -6579,7 +6594,7 @@
     </row>
     <row r="53" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A53" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>4</v>
@@ -6686,7 +6701,7 @@
     </row>
     <row r="54" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A54" s="29" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B54" s="30" t="s">
         <v>4</v>
@@ -6793,7 +6808,7 @@
     </row>
     <row r="55" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A55" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>4</v>
@@ -6900,7 +6915,7 @@
     </row>
     <row r="56" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A56" s="4" t="s">
-        <v>10</v>
+        <v>111</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>4</v>
@@ -7007,7 +7022,7 @@
     </row>
     <row r="57" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A57" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B57" s="4" t="s">
         <v>4</v>
@@ -7114,7 +7129,7 @@
     </row>
     <row r="58" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A58" s="29" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B58" s="30" t="s">
         <v>4</v>
@@ -7221,7 +7236,7 @@
     </row>
     <row r="59" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A59" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B59" s="4" t="s">
         <v>4</v>
@@ -7328,7 +7343,7 @@
     </row>
     <row r="60" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A60" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B60" s="4" t="s">
         <v>4</v>
@@ -7435,7 +7450,7 @@
     </row>
     <row r="61" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A61" s="4" t="s">
-        <v>59</v>
+        <v>112</v>
       </c>
       <c r="B61" s="4" t="s">
         <v>4</v>
@@ -7542,7 +7557,7 @@
     </row>
     <row r="62" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A62" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B62" s="4" t="s">
         <v>4</v>
@@ -7649,7 +7664,7 @@
     </row>
     <row r="63" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A63" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B63" s="4" t="s">
         <v>4</v>
@@ -7756,7 +7771,7 @@
     </row>
     <row r="64" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A64" s="23" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B64" s="24" t="s">
         <v>4</v>
@@ -7863,7 +7878,7 @@
     </row>
     <row r="65" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A65" s="25" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B65" s="25" t="s">
         <v>4</v>
@@ -7970,7 +7985,7 @@
     </row>
     <row r="66" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A66" s="7" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B66" s="8" t="s">
         <v>5</v>
@@ -8076,8 +8091,8 @@
       </c>
     </row>
     <row r="67" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A67" s="4" t="s">
-        <v>16</v>
+      <c r="A67" s="12" t="s">
+        <v>113</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>4</v>
@@ -8184,7 +8199,7 @@
     </row>
     <row r="68" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A68" s="12" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B68" s="4" t="s">
         <v>4</v>
@@ -8291,7 +8306,7 @@
     </row>
     <row r="69" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A69" s="12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B69" s="4" t="s">
         <v>4</v>
@@ -8398,7 +8413,7 @@
     </row>
     <row r="70" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A70" s="29" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B70" s="30" t="s">
         <v>4</v>
@@ -8505,7 +8520,7 @@
     </row>
     <row r="71" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A71" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>4</v>
@@ -8612,7 +8627,7 @@
     </row>
     <row r="72" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A72" s="29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B72" s="30" t="s">
         <v>4</v>
@@ -8719,7 +8734,7 @@
     </row>
     <row r="73" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A73" s="29" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B73" s="30" t="s">
         <v>4</v>
@@ -8826,7 +8841,7 @@
     </row>
     <row r="74" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A74" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B74" s="4" t="s">
         <v>4</v>
@@ -8933,7 +8948,7 @@
     </row>
     <row r="75" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A75" s="4" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B75" s="4" t="s">
         <v>4</v>
@@ -9040,7 +9055,7 @@
     </row>
     <row r="76" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A76" s="4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B76" s="4" t="s">
         <v>4</v>
@@ -9147,7 +9162,7 @@
     </row>
     <row r="77" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A77" s="4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B77" s="4" t="s">
         <v>4</v>
@@ -9254,7 +9269,7 @@
     </row>
     <row r="78" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A78" s="4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B78" s="4" t="s">
         <v>4</v>
@@ -9361,7 +9376,7 @@
     </row>
     <row r="79" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A79" s="12" t="s">
-        <v>64</v>
+        <v>115</v>
       </c>
       <c r="B79" s="4" t="s">
         <v>4</v>
@@ -9468,7 +9483,7 @@
     </row>
     <row r="80" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A80" s="29" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B80" s="30" t="s">
         <v>4</v>
@@ -9575,7 +9590,7 @@
     </row>
     <row r="81" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A81" s="29" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B81" s="30" t="s">
         <v>4</v>
@@ -9682,7 +9697,7 @@
     </row>
     <row r="82" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A82" s="4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B82" s="4" t="s">
         <v>4</v>
@@ -9788,8 +9803,8 @@
       </c>
     </row>
     <row r="83" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A83" s="4" t="s">
-        <v>66</v>
+      <c r="A83" s="12" t="s">
+        <v>116</v>
       </c>
       <c r="B83" s="4" t="s">
         <v>4</v>
@@ -9896,7 +9911,7 @@
     </row>
     <row r="84" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A84" s="4" t="s">
-        <v>68</v>
+        <v>109</v>
       </c>
       <c r="B84" s="4" t="s">
         <v>4</v>
@@ -10003,7 +10018,7 @@
     </row>
     <row r="85" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A85" s="7" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B85" s="8" t="s">
         <v>5</v>
@@ -10110,7 +10125,7 @@
     </row>
     <row r="86" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A86" s="4" t="s">
-        <v>52</v>
+        <v>114</v>
       </c>
       <c r="B86" s="4" t="s">
         <v>4</v>
@@ -10216,8 +10231,8 @@
       </c>
     </row>
     <row r="87" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A87" s="12" t="s">
-        <v>4</v>
+      <c r="A87" s="4" t="s">
+        <v>114</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>11</v>
@@ -10324,7 +10339,7 @@
     </row>
     <row r="88" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A88" s="4" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B88" s="4" t="s">
         <v>4</v>
@@ -10431,7 +10446,7 @@
     </row>
     <row r="89" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A89" s="12" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>4</v>
@@ -10538,7 +10553,7 @@
     </row>
     <row r="90" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A90" s="12" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B90" s="4" t="s">
         <v>4</v>
@@ -10645,7 +10660,7 @@
     </row>
     <row r="91" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A91" s="12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B91" s="4" t="s">
         <v>4</v>
@@ -10752,7 +10767,7 @@
     </row>
     <row r="92" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A92" s="4" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B92" s="4" t="s">
         <v>4</v>
@@ -10859,7 +10874,7 @@
     </row>
     <row r="93" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A93" s="7" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B93" s="8" t="s">
         <v>5</v>
@@ -10966,7 +10981,7 @@
     </row>
     <row r="94" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A94" s="12" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B94" s="4" t="s">
         <v>4</v>
@@ -11073,7 +11088,7 @@
     </row>
     <row r="95" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A95" s="12" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B95" s="4" t="s">
         <v>4</v>
@@ -11180,7 +11195,7 @@
     </row>
     <row r="96" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A96" s="12" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B96" s="4" t="s">
         <v>4</v>
@@ -11287,7 +11302,7 @@
     </row>
     <row r="97" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A97" s="4" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B97" s="4" t="s">
         <v>4</v>
@@ -11394,7 +11409,7 @@
     </row>
     <row r="98" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A98" s="4" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B98" s="4" t="s">
         <v>4</v>
@@ -11501,7 +11516,7 @@
     </row>
     <row r="99" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A99" s="28" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B99" s="28" t="s">
         <v>4</v>
@@ -11608,13 +11623,13 @@
     </row>
     <row r="100" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A100" s="4" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B100" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D100" s="2">
         <v>0</v>
@@ -11715,13 +11730,13 @@
     </row>
     <row r="101" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A101" s="4" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B101" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D101" s="2">
         <v>0</v>
@@ -11822,13 +11837,13 @@
     </row>
     <row r="102" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A102" s="4" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B102" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D102" s="2">
         <v>0</v>
@@ -11929,7 +11944,7 @@
     </row>
     <row r="103" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A103" s="7" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B103" s="8" t="s">
         <v>5</v>
@@ -12036,7 +12051,7 @@
     </row>
     <row r="104" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A104" s="28" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B104" s="28" t="s">
         <v>4</v>
@@ -12143,7 +12158,7 @@
     </row>
     <row r="105" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A105" s="12" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B105" s="4" t="s">
         <v>4</v>
@@ -12250,7 +12265,7 @@
     </row>
     <row r="106" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A106" s="12" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B106" s="4" t="s">
         <v>4</v>
@@ -12357,7 +12372,7 @@
     </row>
     <row r="107" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A107" s="12" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B107" s="4" t="s">
         <v>4</v>
@@ -12464,7 +12479,7 @@
     </row>
     <row r="108" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A108" s="28" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B108" s="28" t="s">
         <v>4</v>
@@ -12571,7 +12586,7 @@
     </row>
     <row r="109" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A109" s="7" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B109" s="8" t="s">
         <v>5</v>
@@ -12678,10 +12693,10 @@
     </row>
     <row r="110" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A110" s="4" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>8</v>
@@ -12785,10 +12800,10 @@
     </row>
     <row r="111" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A111" s="28" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B111" s="28" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>2</v>
@@ -12892,10 +12907,10 @@
     </row>
     <row r="112" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A112" s="4" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B112" s="12" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>2</v>
@@ -12999,10 +13014,10 @@
     </row>
     <row r="113" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A113" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B113" s="12" t="s">
         <v>89</v>
-      </c>
-      <c r="B113" s="12" t="s">
-        <v>93</v>
       </c>
       <c r="C113" s="1" t="s">
         <v>8</v>
@@ -13106,10 +13121,10 @@
     </row>
     <row r="114" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A114" s="4" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B114" s="12" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C114" s="1" t="s">
         <v>2</v>
@@ -13213,10 +13228,10 @@
     </row>
     <row r="115" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A115" s="28" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B115" s="28" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>2</v>
@@ -13320,10 +13335,10 @@
     </row>
     <row r="116" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A116" s="28" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B116" s="28" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>2</v>
@@ -13427,10 +13442,10 @@
     </row>
     <row r="117" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A117" s="4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B117" s="12" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>2</v>
@@ -13534,10 +13549,10 @@
     </row>
     <row r="118" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A118" s="4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B118" s="12" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>2</v>
@@ -13641,10 +13656,10 @@
     </row>
     <row r="119" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A119" s="28" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B119" s="28" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>2</v>
@@ -13748,10 +13763,10 @@
     </row>
     <row r="120" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A120" s="4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C120" s="1" t="s">
         <v>8</v>
@@ -13855,10 +13870,10 @@
     </row>
     <row r="121" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A121" s="28" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B121" s="28" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C121" s="1" t="s">
         <v>2</v>
@@ -13976,7 +13991,7 @@
   <sheetData>
     <row r="1" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>5</v>
@@ -16223,7 +16238,7 @@
     </row>
     <row r="22" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>4</v>
@@ -16330,10 +16345,10 @@
     </row>
     <row r="23" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>7</v>
+        <v>15</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>8</v>
@@ -16437,7 +16452,7 @@
     </row>
     <row r="24" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>11</v>
@@ -16544,7 +16559,7 @@
     </row>
     <row r="25" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A25" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>4</v>
@@ -16651,7 +16666,7 @@
     </row>
     <row r="26" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>11</v>
@@ -16758,7 +16773,7 @@
     </row>
     <row r="27" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B27" s="10" t="s">
         <v>4</v>
@@ -16865,7 +16880,7 @@
     </row>
     <row r="28" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="4" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>11</v>
@@ -16972,7 +16987,7 @@
     </row>
     <row r="29" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="4" t="s">
-        <v>19</v>
+        <v>108</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>4</v>
@@ -17079,7 +17094,7 @@
     </row>
     <row r="30" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B30" s="10" t="s">
         <v>4</v>
@@ -17186,7 +17201,7 @@
     </row>
     <row r="31" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>4</v>
@@ -17293,10 +17308,10 @@
     </row>
     <row r="32" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A32" s="4" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>8</v>
@@ -17400,7 +17415,7 @@
     </row>
     <row r="33" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A33" s="16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>4</v>
@@ -17507,7 +17522,7 @@
     </row>
     <row r="34" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="16" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>4</v>
@@ -17614,7 +17629,7 @@
     </row>
     <row r="35" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A35" s="14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B35" s="10" t="s">
         <v>4</v>
@@ -17721,7 +17736,7 @@
     </row>
     <row r="36" spans="1:35" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A36" s="17" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="B36" s="18" t="s">
         <v>11</v>
@@ -17828,7 +17843,7 @@
     </row>
     <row r="37" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="7" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B37" s="8" t="s">
         <v>5</v>
@@ -17935,7 +17950,7 @@
     </row>
     <row r="38" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A38" s="29" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B38" s="30" t="s">
         <v>4</v>
@@ -18042,7 +18057,7 @@
     </row>
     <row r="39" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A39" s="22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>4</v>
@@ -18149,7 +18164,7 @@
     </row>
     <row r="40" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A40" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>4</v>
@@ -18256,7 +18271,7 @@
     </row>
     <row r="41" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A41" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>4</v>
@@ -18363,7 +18378,7 @@
     </row>
     <row r="42" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="29" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B42" s="30" t="s">
         <v>4</v>
@@ -18470,7 +18485,7 @@
     </row>
     <row r="43" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A43" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>4</v>
@@ -18577,7 +18592,7 @@
     </row>
     <row r="44" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A44" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>4</v>
@@ -18684,7 +18699,7 @@
     </row>
     <row r="45" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A45" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B45" s="4" t="s">
         <v>4</v>
@@ -18791,7 +18806,7 @@
     </row>
     <row r="46" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A46" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B46" s="4" t="s">
         <v>4</v>
@@ -18898,7 +18913,7 @@
     </row>
     <row r="47" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A47" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>4</v>
@@ -19005,7 +19020,7 @@
     </row>
     <row r="48" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A48" s="23" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B48" s="24" t="s">
         <v>4</v>
@@ -19112,7 +19127,7 @@
     </row>
     <row r="49" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A49" s="29" t="s">
-        <v>58</v>
+        <v>110</v>
       </c>
       <c r="B49" s="30" t="s">
         <v>4</v>
@@ -19219,7 +19234,7 @@
     </row>
     <row r="50" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A50" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>4</v>
@@ -19326,7 +19341,7 @@
     </row>
     <row r="51" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A51" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>4</v>
@@ -19433,7 +19448,7 @@
     </row>
     <row r="52" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A52" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>4</v>
@@ -19540,7 +19555,7 @@
     </row>
     <row r="53" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A53" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>4</v>
@@ -19647,7 +19662,7 @@
     </row>
     <row r="54" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A54" s="29" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B54" s="30" t="s">
         <v>4</v>
@@ -19754,7 +19769,7 @@
     </row>
     <row r="55" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A55" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>4</v>
@@ -19861,7 +19876,7 @@
     </row>
     <row r="56" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A56" s="4" t="s">
-        <v>10</v>
+        <v>111</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>4</v>
@@ -19968,7 +19983,7 @@
     </row>
     <row r="57" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A57" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B57" s="4" t="s">
         <v>4</v>
@@ -20075,7 +20090,7 @@
     </row>
     <row r="58" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A58" s="29" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B58" s="30" t="s">
         <v>4</v>
@@ -20182,7 +20197,7 @@
     </row>
     <row r="59" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A59" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B59" s="4" t="s">
         <v>4</v>
@@ -20289,7 +20304,7 @@
     </row>
     <row r="60" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A60" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B60" s="4" t="s">
         <v>4</v>
@@ -20396,7 +20411,7 @@
     </row>
     <row r="61" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A61" s="4" t="s">
-        <v>59</v>
+        <v>112</v>
       </c>
       <c r="B61" s="4" t="s">
         <v>4</v>
@@ -20503,7 +20518,7 @@
     </row>
     <row r="62" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A62" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B62" s="4" t="s">
         <v>4</v>
@@ -20610,7 +20625,7 @@
     </row>
     <row r="63" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A63" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B63" s="4" t="s">
         <v>4</v>
@@ -20717,7 +20732,7 @@
     </row>
     <row r="64" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A64" s="23" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B64" s="24" t="s">
         <v>4</v>
@@ -20824,7 +20839,7 @@
     </row>
     <row r="65" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A65" s="25" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B65" s="25" t="s">
         <v>4</v>
@@ -20931,7 +20946,7 @@
     </row>
     <row r="66" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A66" s="7" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B66" s="8" t="s">
         <v>5</v>
@@ -21037,8 +21052,8 @@
       </c>
     </row>
     <row r="67" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A67" s="4" t="s">
-        <v>16</v>
+      <c r="A67" s="12" t="s">
+        <v>113</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>4</v>
@@ -21145,7 +21160,7 @@
     </row>
     <row r="68" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A68" s="12" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B68" s="4" t="s">
         <v>4</v>
@@ -21252,7 +21267,7 @@
     </row>
     <row r="69" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A69" s="12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B69" s="4" t="s">
         <v>4</v>
@@ -21359,7 +21374,7 @@
     </row>
     <row r="70" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A70" s="29" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B70" s="30" t="s">
         <v>4</v>
@@ -21466,7 +21481,7 @@
     </row>
     <row r="71" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A71" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>4</v>
@@ -21573,7 +21588,7 @@
     </row>
     <row r="72" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A72" s="29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B72" s="30" t="s">
         <v>4</v>
@@ -21680,7 +21695,7 @@
     </row>
     <row r="73" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A73" s="29" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B73" s="30" t="s">
         <v>4</v>
@@ -21787,7 +21802,7 @@
     </row>
     <row r="74" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A74" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B74" s="4" t="s">
         <v>4</v>
@@ -21894,7 +21909,7 @@
     </row>
     <row r="75" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A75" s="4" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B75" s="4" t="s">
         <v>4</v>
@@ -22001,7 +22016,7 @@
     </row>
     <row r="76" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A76" s="4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B76" s="4" t="s">
         <v>4</v>
@@ -22108,7 +22123,7 @@
     </row>
     <row r="77" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A77" s="4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B77" s="4" t="s">
         <v>4</v>
@@ -22215,7 +22230,7 @@
     </row>
     <row r="78" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A78" s="4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B78" s="4" t="s">
         <v>4</v>
@@ -22322,7 +22337,7 @@
     </row>
     <row r="79" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A79" s="12" t="s">
-        <v>64</v>
+        <v>115</v>
       </c>
       <c r="B79" s="4" t="s">
         <v>4</v>
@@ -22429,7 +22444,7 @@
     </row>
     <row r="80" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A80" s="29" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B80" s="30" t="s">
         <v>4</v>
@@ -22536,7 +22551,7 @@
     </row>
     <row r="81" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A81" s="29" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B81" s="30" t="s">
         <v>4</v>
@@ -22643,7 +22658,7 @@
     </row>
     <row r="82" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A82" s="4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B82" s="4" t="s">
         <v>4</v>
@@ -22749,8 +22764,8 @@
       </c>
     </row>
     <row r="83" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A83" s="4" t="s">
-        <v>66</v>
+      <c r="A83" s="12" t="s">
+        <v>116</v>
       </c>
       <c r="B83" s="4" t="s">
         <v>4</v>
@@ -22857,7 +22872,7 @@
     </row>
     <row r="84" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A84" s="4" t="s">
-        <v>68</v>
+        <v>109</v>
       </c>
       <c r="B84" s="4" t="s">
         <v>4</v>
@@ -22964,7 +22979,7 @@
     </row>
     <row r="85" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A85" s="7" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B85" s="8" t="s">
         <v>5</v>
@@ -23071,7 +23086,7 @@
     </row>
     <row r="86" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A86" s="4" t="s">
-        <v>52</v>
+        <v>114</v>
       </c>
       <c r="B86" s="4" t="s">
         <v>4</v>
@@ -23177,8 +23192,8 @@
       </c>
     </row>
     <row r="87" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A87" s="12" t="s">
-        <v>4</v>
+      <c r="A87" s="4" t="s">
+        <v>114</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>11</v>
@@ -23285,7 +23300,7 @@
     </row>
     <row r="88" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A88" s="4" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B88" s="4" t="s">
         <v>4</v>
@@ -23392,7 +23407,7 @@
     </row>
     <row r="89" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A89" s="12" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>4</v>
@@ -23499,7 +23514,7 @@
     </row>
     <row r="90" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A90" s="12" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B90" s="4" t="s">
         <v>4</v>
@@ -23606,7 +23621,7 @@
     </row>
     <row r="91" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A91" s="12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B91" s="4" t="s">
         <v>4</v>
@@ -23713,7 +23728,7 @@
     </row>
     <row r="92" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A92" s="4" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B92" s="4" t="s">
         <v>4</v>
@@ -23820,7 +23835,7 @@
     </row>
     <row r="93" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A93" s="7" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B93" s="8" t="s">
         <v>5</v>
@@ -23927,7 +23942,7 @@
     </row>
     <row r="94" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A94" s="12" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B94" s="4" t="s">
         <v>4</v>
@@ -24034,7 +24049,7 @@
     </row>
     <row r="95" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A95" s="12" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B95" s="4" t="s">
         <v>4</v>
@@ -24141,7 +24156,7 @@
     </row>
     <row r="96" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A96" s="12" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B96" s="4" t="s">
         <v>4</v>
@@ -24248,7 +24263,7 @@
     </row>
     <row r="97" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A97" s="4" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B97" s="4" t="s">
         <v>4</v>
@@ -24355,7 +24370,7 @@
     </row>
     <row r="98" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A98" s="4" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B98" s="4" t="s">
         <v>4</v>
@@ -24462,7 +24477,7 @@
     </row>
     <row r="99" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A99" s="28" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B99" s="28" t="s">
         <v>4</v>
@@ -24569,13 +24584,13 @@
     </row>
     <row r="100" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A100" s="4" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B100" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D100" s="2">
         <v>0</v>
@@ -24676,13 +24691,13 @@
     </row>
     <row r="101" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A101" s="4" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B101" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D101" s="2">
         <v>0</v>
@@ -24783,13 +24798,13 @@
     </row>
     <row r="102" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A102" s="4" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B102" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D102" s="2">
         <v>0</v>
@@ -24890,7 +24905,7 @@
     </row>
     <row r="103" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A103" s="7" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B103" s="8" t="s">
         <v>5</v>
@@ -24997,7 +25012,7 @@
     </row>
     <row r="104" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A104" s="28" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B104" s="28" t="s">
         <v>4</v>
@@ -25104,7 +25119,7 @@
     </row>
     <row r="105" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A105" s="12" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B105" s="4" t="s">
         <v>4</v>
@@ -25211,7 +25226,7 @@
     </row>
     <row r="106" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A106" s="12" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B106" s="4" t="s">
         <v>4</v>
@@ -25318,7 +25333,7 @@
     </row>
     <row r="107" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A107" s="12" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B107" s="4" t="s">
         <v>4</v>
@@ -25425,7 +25440,7 @@
     </row>
     <row r="108" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A108" s="28" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B108" s="28" t="s">
         <v>4</v>
@@ -25532,7 +25547,7 @@
     </row>
     <row r="109" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A109" s="7" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B109" s="8" t="s">
         <v>5</v>
@@ -25639,10 +25654,10 @@
     </row>
     <row r="110" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A110" s="4" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>8</v>
@@ -25746,10 +25761,10 @@
     </row>
     <row r="111" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A111" s="28" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B111" s="28" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>2</v>
@@ -25853,10 +25868,10 @@
     </row>
     <row r="112" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A112" s="4" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B112" s="12" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>2</v>
@@ -25960,10 +25975,10 @@
     </row>
     <row r="113" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A113" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B113" s="12" t="s">
         <v>89</v>
-      </c>
-      <c r="B113" s="12" t="s">
-        <v>93</v>
       </c>
       <c r="C113" s="1" t="s">
         <v>8</v>
@@ -26067,10 +26082,10 @@
     </row>
     <row r="114" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A114" s="4" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B114" s="12" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C114" s="1" t="s">
         <v>2</v>
@@ -26174,10 +26189,10 @@
     </row>
     <row r="115" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A115" s="28" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B115" s="28" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>2</v>
@@ -26281,10 +26296,10 @@
     </row>
     <row r="116" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A116" s="28" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B116" s="28" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>2</v>
@@ -26388,10 +26403,10 @@
     </row>
     <row r="117" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A117" s="4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B117" s="12" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>2</v>
@@ -26495,10 +26510,10 @@
     </row>
     <row r="118" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A118" s="4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B118" s="12" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>2</v>
@@ -26602,10 +26617,10 @@
     </row>
     <row r="119" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A119" s="28" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B119" s="28" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>2</v>
@@ -26709,10 +26724,10 @@
     </row>
     <row r="120" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A120" s="4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C120" s="1" t="s">
         <v>8</v>
@@ -26816,10 +26831,10 @@
     </row>
     <row r="121" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A121" s="28" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B121" s="28" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C121" s="1" t="s">
         <v>2</v>
@@ -26937,7 +26952,7 @@
   <sheetData>
     <row r="1" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>5</v>
@@ -29184,7 +29199,7 @@
     </row>
     <row r="22" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>4</v>
@@ -29291,10 +29306,10 @@
     </row>
     <row r="23" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>7</v>
+        <v>15</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>8</v>
@@ -29398,7 +29413,7 @@
     </row>
     <row r="24" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>11</v>
@@ -29505,7 +29520,7 @@
     </row>
     <row r="25" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A25" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>4</v>
@@ -29612,7 +29627,7 @@
     </row>
     <row r="26" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>11</v>
@@ -29719,7 +29734,7 @@
     </row>
     <row r="27" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B27" s="10" t="s">
         <v>4</v>
@@ -29826,7 +29841,7 @@
     </row>
     <row r="28" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="4" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>11</v>
@@ -29933,7 +29948,7 @@
     </row>
     <row r="29" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="4" t="s">
-        <v>19</v>
+        <v>108</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>4</v>
@@ -30040,7 +30055,7 @@
     </row>
     <row r="30" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B30" s="10" t="s">
         <v>4</v>
@@ -30147,7 +30162,7 @@
     </row>
     <row r="31" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>4</v>
@@ -30254,10 +30269,10 @@
     </row>
     <row r="32" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A32" s="4" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>8</v>
@@ -30361,7 +30376,7 @@
     </row>
     <row r="33" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A33" s="16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>4</v>
@@ -30468,7 +30483,7 @@
     </row>
     <row r="34" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="16" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>4</v>
@@ -30575,7 +30590,7 @@
     </row>
     <row r="35" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A35" s="14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B35" s="10" t="s">
         <v>4</v>
@@ -30682,7 +30697,7 @@
     </row>
     <row r="36" spans="1:35" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A36" s="17" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="B36" s="18" t="s">
         <v>11</v>
@@ -30789,7 +30804,7 @@
     </row>
     <row r="37" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="7" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B37" s="8" t="s">
         <v>5</v>
@@ -30896,7 +30911,7 @@
     </row>
     <row r="38" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A38" s="29" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B38" s="30" t="s">
         <v>4</v>
@@ -31003,7 +31018,7 @@
     </row>
     <row r="39" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A39" s="22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>4</v>
@@ -31110,7 +31125,7 @@
     </row>
     <row r="40" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A40" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>4</v>
@@ -31217,7 +31232,7 @@
     </row>
     <row r="41" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A41" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>4</v>
@@ -31324,7 +31339,7 @@
     </row>
     <row r="42" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="29" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B42" s="30" t="s">
         <v>4</v>
@@ -31431,7 +31446,7 @@
     </row>
     <row r="43" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A43" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>4</v>
@@ -31538,7 +31553,7 @@
     </row>
     <row r="44" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A44" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>4</v>
@@ -31645,7 +31660,7 @@
     </row>
     <row r="45" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A45" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B45" s="4" t="s">
         <v>4</v>
@@ -31752,7 +31767,7 @@
     </row>
     <row r="46" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A46" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B46" s="4" t="s">
         <v>4</v>
@@ -31859,7 +31874,7 @@
     </row>
     <row r="47" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A47" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>4</v>
@@ -31966,7 +31981,7 @@
     </row>
     <row r="48" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A48" s="23" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B48" s="24" t="s">
         <v>4</v>
@@ -32073,7 +32088,7 @@
     </row>
     <row r="49" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A49" s="29" t="s">
-        <v>58</v>
+        <v>110</v>
       </c>
       <c r="B49" s="30" t="s">
         <v>4</v>
@@ -32180,7 +32195,7 @@
     </row>
     <row r="50" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A50" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>4</v>
@@ -32287,7 +32302,7 @@
     </row>
     <row r="51" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A51" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>4</v>
@@ -32394,7 +32409,7 @@
     </row>
     <row r="52" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A52" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>4</v>
@@ -32501,7 +32516,7 @@
     </row>
     <row r="53" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A53" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>4</v>
@@ -32608,7 +32623,7 @@
     </row>
     <row r="54" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A54" s="29" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B54" s="30" t="s">
         <v>4</v>
@@ -32715,7 +32730,7 @@
     </row>
     <row r="55" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A55" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>4</v>
@@ -32822,7 +32837,7 @@
     </row>
     <row r="56" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A56" s="4" t="s">
-        <v>10</v>
+        <v>111</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>4</v>
@@ -32929,7 +32944,7 @@
     </row>
     <row r="57" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A57" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B57" s="4" t="s">
         <v>4</v>
@@ -33036,7 +33051,7 @@
     </row>
     <row r="58" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A58" s="29" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B58" s="30" t="s">
         <v>4</v>
@@ -33143,7 +33158,7 @@
     </row>
     <row r="59" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A59" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B59" s="4" t="s">
         <v>4</v>
@@ -33250,7 +33265,7 @@
     </row>
     <row r="60" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A60" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B60" s="4" t="s">
         <v>4</v>
@@ -33357,7 +33372,7 @@
     </row>
     <row r="61" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A61" s="4" t="s">
-        <v>59</v>
+        <v>112</v>
       </c>
       <c r="B61" s="4" t="s">
         <v>4</v>
@@ -33464,7 +33479,7 @@
     </row>
     <row r="62" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A62" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B62" s="4" t="s">
         <v>4</v>
@@ -33571,7 +33586,7 @@
     </row>
     <row r="63" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A63" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B63" s="4" t="s">
         <v>4</v>
@@ -33678,7 +33693,7 @@
     </row>
     <row r="64" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A64" s="23" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B64" s="24" t="s">
         <v>4</v>
@@ -33785,7 +33800,7 @@
     </row>
     <row r="65" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A65" s="25" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B65" s="25" t="s">
         <v>4</v>
@@ -33892,7 +33907,7 @@
     </row>
     <row r="66" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A66" s="7" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B66" s="8" t="s">
         <v>5</v>
@@ -33998,8 +34013,8 @@
       </c>
     </row>
     <row r="67" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A67" s="4" t="s">
-        <v>16</v>
+      <c r="A67" s="12" t="s">
+        <v>113</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>4</v>
@@ -34106,7 +34121,7 @@
     </row>
     <row r="68" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A68" s="12" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B68" s="4" t="s">
         <v>4</v>
@@ -34213,7 +34228,7 @@
     </row>
     <row r="69" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A69" s="12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B69" s="4" t="s">
         <v>4</v>
@@ -34320,7 +34335,7 @@
     </row>
     <row r="70" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A70" s="29" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B70" s="30" t="s">
         <v>4</v>
@@ -34427,7 +34442,7 @@
     </row>
     <row r="71" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A71" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>4</v>
@@ -34534,7 +34549,7 @@
     </row>
     <row r="72" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A72" s="29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B72" s="30" t="s">
         <v>4</v>
@@ -34641,7 +34656,7 @@
     </row>
     <row r="73" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A73" s="29" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B73" s="30" t="s">
         <v>4</v>
@@ -34748,7 +34763,7 @@
     </row>
     <row r="74" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A74" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B74" s="4" t="s">
         <v>4</v>
@@ -34855,7 +34870,7 @@
     </row>
     <row r="75" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A75" s="4" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B75" s="4" t="s">
         <v>4</v>
@@ -34962,7 +34977,7 @@
     </row>
     <row r="76" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A76" s="4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B76" s="4" t="s">
         <v>4</v>
@@ -35069,7 +35084,7 @@
     </row>
     <row r="77" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A77" s="4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B77" s="4" t="s">
         <v>4</v>
@@ -35176,7 +35191,7 @@
     </row>
     <row r="78" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A78" s="4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B78" s="4" t="s">
         <v>4</v>
@@ -35283,7 +35298,7 @@
     </row>
     <row r="79" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A79" s="12" t="s">
-        <v>64</v>
+        <v>115</v>
       </c>
       <c r="B79" s="4" t="s">
         <v>4</v>
@@ -35390,7 +35405,7 @@
     </row>
     <row r="80" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A80" s="29" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B80" s="30" t="s">
         <v>4</v>
@@ -35497,7 +35512,7 @@
     </row>
     <row r="81" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A81" s="29" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B81" s="30" t="s">
         <v>4</v>
@@ -35604,7 +35619,7 @@
     </row>
     <row r="82" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A82" s="4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B82" s="4" t="s">
         <v>4</v>
@@ -35710,8 +35725,8 @@
       </c>
     </row>
     <row r="83" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A83" s="4" t="s">
-        <v>66</v>
+      <c r="A83" s="12" t="s">
+        <v>116</v>
       </c>
       <c r="B83" s="4" t="s">
         <v>4</v>
@@ -35818,7 +35833,7 @@
     </row>
     <row r="84" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A84" s="4" t="s">
-        <v>68</v>
+        <v>109</v>
       </c>
       <c r="B84" s="4" t="s">
         <v>4</v>
@@ -35925,7 +35940,7 @@
     </row>
     <row r="85" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A85" s="7" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B85" s="8" t="s">
         <v>5</v>
@@ -36032,7 +36047,7 @@
     </row>
     <row r="86" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A86" s="4" t="s">
-        <v>52</v>
+        <v>114</v>
       </c>
       <c r="B86" s="4" t="s">
         <v>4</v>
@@ -36138,8 +36153,8 @@
       </c>
     </row>
     <row r="87" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A87" s="12" t="s">
-        <v>4</v>
+      <c r="A87" s="4" t="s">
+        <v>114</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>11</v>
@@ -36246,7 +36261,7 @@
     </row>
     <row r="88" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A88" s="4" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B88" s="4" t="s">
         <v>4</v>
@@ -36353,7 +36368,7 @@
     </row>
     <row r="89" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A89" s="12" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>4</v>
@@ -36460,7 +36475,7 @@
     </row>
     <row r="90" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A90" s="12" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B90" s="4" t="s">
         <v>4</v>
@@ -36567,7 +36582,7 @@
     </row>
     <row r="91" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A91" s="12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B91" s="4" t="s">
         <v>4</v>
@@ -36674,7 +36689,7 @@
     </row>
     <row r="92" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A92" s="4" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B92" s="4" t="s">
         <v>4</v>
@@ -36781,7 +36796,7 @@
     </row>
     <row r="93" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A93" s="7" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B93" s="8" t="s">
         <v>5</v>
@@ -36888,7 +36903,7 @@
     </row>
     <row r="94" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A94" s="12" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B94" s="4" t="s">
         <v>4</v>
@@ -36995,7 +37010,7 @@
     </row>
     <row r="95" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A95" s="12" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B95" s="4" t="s">
         <v>4</v>
@@ -37102,7 +37117,7 @@
     </row>
     <row r="96" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A96" s="12" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B96" s="4" t="s">
         <v>4</v>
@@ -37209,7 +37224,7 @@
     </row>
     <row r="97" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A97" s="4" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B97" s="4" t="s">
         <v>4</v>
@@ -37316,7 +37331,7 @@
     </row>
     <row r="98" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A98" s="4" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B98" s="4" t="s">
         <v>4</v>
@@ -37423,7 +37438,7 @@
     </row>
     <row r="99" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A99" s="28" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B99" s="28" t="s">
         <v>4</v>
@@ -37530,13 +37545,13 @@
     </row>
     <row r="100" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A100" s="4" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B100" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D100" s="2">
         <v>0</v>
@@ -37637,13 +37652,13 @@
     </row>
     <row r="101" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A101" s="4" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B101" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D101" s="2">
         <v>0</v>
@@ -37744,13 +37759,13 @@
     </row>
     <row r="102" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A102" s="4" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B102" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D102" s="2">
         <v>0</v>
@@ -37851,7 +37866,7 @@
     </row>
     <row r="103" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A103" s="7" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B103" s="8" t="s">
         <v>5</v>
@@ -37958,7 +37973,7 @@
     </row>
     <row r="104" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A104" s="28" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B104" s="28" t="s">
         <v>4</v>
@@ -38065,7 +38080,7 @@
     </row>
     <row r="105" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A105" s="12" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B105" s="4" t="s">
         <v>4</v>
@@ -38172,7 +38187,7 @@
     </row>
     <row r="106" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A106" s="12" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B106" s="4" t="s">
         <v>4</v>
@@ -38279,7 +38294,7 @@
     </row>
     <row r="107" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A107" s="12" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B107" s="4" t="s">
         <v>4</v>
@@ -38386,7 +38401,7 @@
     </row>
     <row r="108" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A108" s="28" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B108" s="28" t="s">
         <v>4</v>
@@ -38493,7 +38508,7 @@
     </row>
     <row r="109" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A109" s="7" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B109" s="8" t="s">
         <v>5</v>
@@ -38600,10 +38615,10 @@
     </row>
     <row r="110" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A110" s="4" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>8</v>
@@ -38707,10 +38722,10 @@
     </row>
     <row r="111" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A111" s="28" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B111" s="28" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>2</v>
@@ -38814,10 +38829,10 @@
     </row>
     <row r="112" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A112" s="4" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B112" s="12" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>2</v>
@@ -38921,10 +38936,10 @@
     </row>
     <row r="113" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A113" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B113" s="12" t="s">
         <v>89</v>
-      </c>
-      <c r="B113" s="12" t="s">
-        <v>93</v>
       </c>
       <c r="C113" s="1" t="s">
         <v>8</v>
@@ -39028,10 +39043,10 @@
     </row>
     <row r="114" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A114" s="4" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B114" s="12" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C114" s="1" t="s">
         <v>2</v>
@@ -39135,10 +39150,10 @@
     </row>
     <row r="115" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A115" s="28" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B115" s="28" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>2</v>
@@ -39242,10 +39257,10 @@
     </row>
     <row r="116" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A116" s="28" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B116" s="28" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>2</v>
@@ -39349,10 +39364,10 @@
     </row>
     <row r="117" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A117" s="4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B117" s="12" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>2</v>
@@ -39456,10 +39471,10 @@
     </row>
     <row r="118" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A118" s="4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B118" s="12" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>2</v>
@@ -39563,10 +39578,10 @@
     </row>
     <row r="119" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A119" s="28" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B119" s="28" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>2</v>
@@ -39670,10 +39685,10 @@
     </row>
     <row r="120" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A120" s="4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C120" s="1" t="s">
         <v>8</v>
@@ -39777,10 +39792,10 @@
     </row>
     <row r="121" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A121" s="28" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B121" s="28" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C121" s="1" t="s">
         <v>2</v>
@@ -39884,7 +39899,7 @@
     </row>
     <row r="122" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A122" s="7" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B122" s="8" t="s">
         <v>5</v>
@@ -39991,7 +40006,7 @@
     </row>
     <row r="123" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A123" s="12" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B123" s="4" t="s">
         <v>4</v>
@@ -40098,7 +40113,7 @@
     </row>
     <row r="124" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A124" s="12" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B124" s="4" t="s">
         <v>4</v>
@@ -40205,13 +40220,13 @@
     </row>
     <row r="125" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A125" s="12" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B125" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D125" s="2">
         <v>0</v>
@@ -40312,7 +40327,7 @@
     </row>
     <row r="126" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A126" s="23" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B126" s="24" t="s">
         <v>4</v>
@@ -40434,7 +40449,7 @@
   <sheetData>
     <row r="1" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>5</v>
@@ -42681,7 +42696,7 @@
     </row>
     <row r="22" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>4</v>
@@ -42788,10 +42803,10 @@
     </row>
     <row r="23" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>7</v>
+        <v>15</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>8</v>
@@ -42895,7 +42910,7 @@
     </row>
     <row r="24" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>11</v>
@@ -43002,7 +43017,7 @@
     </row>
     <row r="25" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A25" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>4</v>
@@ -43109,7 +43124,7 @@
     </row>
     <row r="26" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>11</v>
@@ -43216,7 +43231,7 @@
     </row>
     <row r="27" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B27" s="10" t="s">
         <v>4</v>
@@ -43323,7 +43338,7 @@
     </row>
     <row r="28" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="4" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>11</v>
@@ -43430,7 +43445,7 @@
     </row>
     <row r="29" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="4" t="s">
-        <v>19</v>
+        <v>108</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>4</v>
@@ -43537,7 +43552,7 @@
     </row>
     <row r="30" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B30" s="10" t="s">
         <v>4</v>
@@ -43644,7 +43659,7 @@
     </row>
     <row r="31" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>4</v>
@@ -43751,10 +43766,10 @@
     </row>
     <row r="32" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A32" s="4" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>8</v>
@@ -43858,7 +43873,7 @@
     </row>
     <row r="33" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A33" s="16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>4</v>
@@ -43965,7 +43980,7 @@
     </row>
     <row r="34" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="16" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>4</v>
@@ -44072,7 +44087,7 @@
     </row>
     <row r="35" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A35" s="14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B35" s="10" t="s">
         <v>4</v>
@@ -44179,7 +44194,7 @@
     </row>
     <row r="36" spans="1:35" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A36" s="17" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="B36" s="18" t="s">
         <v>11</v>
@@ -44286,7 +44301,7 @@
     </row>
     <row r="37" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="7" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B37" s="8" t="s">
         <v>5</v>
@@ -44393,7 +44408,7 @@
     </row>
     <row r="38" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A38" s="29" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B38" s="30" t="s">
         <v>4</v>
@@ -44500,7 +44515,7 @@
     </row>
     <row r="39" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A39" s="22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>4</v>
@@ -44607,7 +44622,7 @@
     </row>
     <row r="40" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A40" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>4</v>
@@ -44714,7 +44729,7 @@
     </row>
     <row r="41" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A41" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>4</v>
@@ -44821,7 +44836,7 @@
     </row>
     <row r="42" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="29" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B42" s="30" t="s">
         <v>4</v>
@@ -44928,7 +44943,7 @@
     </row>
     <row r="43" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A43" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>4</v>
@@ -45035,7 +45050,7 @@
     </row>
     <row r="44" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A44" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>4</v>
@@ -45142,7 +45157,7 @@
     </row>
     <row r="45" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A45" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B45" s="4" t="s">
         <v>4</v>
@@ -45249,7 +45264,7 @@
     </row>
     <row r="46" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A46" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B46" s="4" t="s">
         <v>4</v>
@@ -45356,7 +45371,7 @@
     </row>
     <row r="47" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A47" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>4</v>
@@ -45463,7 +45478,7 @@
     </row>
     <row r="48" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A48" s="23" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B48" s="24" t="s">
         <v>4</v>
@@ -45570,7 +45585,7 @@
     </row>
     <row r="49" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A49" s="29" t="s">
-        <v>58</v>
+        <v>110</v>
       </c>
       <c r="B49" s="30" t="s">
         <v>4</v>
@@ -45677,7 +45692,7 @@
     </row>
     <row r="50" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A50" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>4</v>
@@ -45784,7 +45799,7 @@
     </row>
     <row r="51" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A51" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>4</v>
@@ -45891,7 +45906,7 @@
     </row>
     <row r="52" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A52" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>4</v>
@@ -45998,7 +46013,7 @@
     </row>
     <row r="53" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A53" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>4</v>
@@ -46105,7 +46120,7 @@
     </row>
     <row r="54" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A54" s="29" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B54" s="30" t="s">
         <v>4</v>
@@ -46212,7 +46227,7 @@
     </row>
     <row r="55" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A55" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>4</v>
@@ -46319,7 +46334,7 @@
     </row>
     <row r="56" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A56" s="4" t="s">
-        <v>10</v>
+        <v>111</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>4</v>
@@ -46426,7 +46441,7 @@
     </row>
     <row r="57" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A57" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B57" s="4" t="s">
         <v>4</v>
@@ -46533,7 +46548,7 @@
     </row>
     <row r="58" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A58" s="29" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B58" s="30" t="s">
         <v>4</v>
@@ -46640,7 +46655,7 @@
     </row>
     <row r="59" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A59" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B59" s="4" t="s">
         <v>4</v>
@@ -46747,7 +46762,7 @@
     </row>
     <row r="60" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A60" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B60" s="4" t="s">
         <v>4</v>
@@ -46854,7 +46869,7 @@
     </row>
     <row r="61" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A61" s="4" t="s">
-        <v>59</v>
+        <v>112</v>
       </c>
       <c r="B61" s="4" t="s">
         <v>4</v>
@@ -46961,7 +46976,7 @@
     </row>
     <row r="62" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A62" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B62" s="4" t="s">
         <v>4</v>
@@ -47068,7 +47083,7 @@
     </row>
     <row r="63" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A63" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B63" s="4" t="s">
         <v>4</v>
@@ -47175,7 +47190,7 @@
     </row>
     <row r="64" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A64" s="23" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B64" s="24" t="s">
         <v>4</v>
@@ -47282,7 +47297,7 @@
     </row>
     <row r="65" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A65" s="25" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B65" s="25" t="s">
         <v>4</v>
@@ -47389,7 +47404,7 @@
     </row>
     <row r="66" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A66" s="7" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B66" s="8" t="s">
         <v>5</v>
@@ -47495,8 +47510,8 @@
       </c>
     </row>
     <row r="67" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A67" s="4" t="s">
-        <v>16</v>
+      <c r="A67" s="12" t="s">
+        <v>113</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>4</v>
@@ -47603,7 +47618,7 @@
     </row>
     <row r="68" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A68" s="12" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B68" s="4" t="s">
         <v>4</v>
@@ -47710,7 +47725,7 @@
     </row>
     <row r="69" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A69" s="12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B69" s="4" t="s">
         <v>4</v>
@@ -47817,7 +47832,7 @@
     </row>
     <row r="70" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A70" s="29" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B70" s="30" t="s">
         <v>4</v>
@@ -47924,7 +47939,7 @@
     </row>
     <row r="71" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A71" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>4</v>
@@ -48031,7 +48046,7 @@
     </row>
     <row r="72" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A72" s="29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B72" s="30" t="s">
         <v>4</v>
@@ -48138,7 +48153,7 @@
     </row>
     <row r="73" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A73" s="29" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B73" s="30" t="s">
         <v>4</v>
@@ -48245,7 +48260,7 @@
     </row>
     <row r="74" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A74" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B74" s="4" t="s">
         <v>4</v>
@@ -48352,7 +48367,7 @@
     </row>
     <row r="75" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A75" s="4" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B75" s="4" t="s">
         <v>4</v>
@@ -48459,7 +48474,7 @@
     </row>
     <row r="76" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A76" s="4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B76" s="4" t="s">
         <v>4</v>
@@ -48566,7 +48581,7 @@
     </row>
     <row r="77" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A77" s="4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B77" s="4" t="s">
         <v>4</v>
@@ -48673,7 +48688,7 @@
     </row>
     <row r="78" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A78" s="4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B78" s="4" t="s">
         <v>4</v>
@@ -48780,7 +48795,7 @@
     </row>
     <row r="79" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A79" s="12" t="s">
-        <v>64</v>
+        <v>115</v>
       </c>
       <c r="B79" s="4" t="s">
         <v>4</v>
@@ -48887,7 +48902,7 @@
     </row>
     <row r="80" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A80" s="29" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B80" s="30" t="s">
         <v>4</v>
@@ -48994,7 +49009,7 @@
     </row>
     <row r="81" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A81" s="29" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B81" s="30" t="s">
         <v>4</v>
@@ -49101,7 +49116,7 @@
     </row>
     <row r="82" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A82" s="4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B82" s="4" t="s">
         <v>4</v>
@@ -49207,8 +49222,8 @@
       </c>
     </row>
     <row r="83" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A83" s="4" t="s">
-        <v>66</v>
+      <c r="A83" s="12" t="s">
+        <v>116</v>
       </c>
       <c r="B83" s="4" t="s">
         <v>4</v>
@@ -49315,7 +49330,7 @@
     </row>
     <row r="84" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A84" s="4" t="s">
-        <v>68</v>
+        <v>109</v>
       </c>
       <c r="B84" s="4" t="s">
         <v>4</v>
@@ -49422,7 +49437,7 @@
     </row>
     <row r="85" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A85" s="7" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B85" s="8" t="s">
         <v>5</v>
@@ -49529,7 +49544,7 @@
     </row>
     <row r="86" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A86" s="4" t="s">
-        <v>52</v>
+        <v>114</v>
       </c>
       <c r="B86" s="4" t="s">
         <v>4</v>
@@ -49635,8 +49650,8 @@
       </c>
     </row>
     <row r="87" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A87" s="12" t="s">
-        <v>4</v>
+      <c r="A87" s="4" t="s">
+        <v>114</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>11</v>
@@ -49743,7 +49758,7 @@
     </row>
     <row r="88" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A88" s="4" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B88" s="4" t="s">
         <v>4</v>
@@ -49850,7 +49865,7 @@
     </row>
     <row r="89" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A89" s="12" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>4</v>
@@ -49957,7 +49972,7 @@
     </row>
     <row r="90" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A90" s="12" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B90" s="4" t="s">
         <v>4</v>
@@ -50064,7 +50079,7 @@
     </row>
     <row r="91" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A91" s="12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B91" s="4" t="s">
         <v>4</v>
@@ -50171,7 +50186,7 @@
     </row>
     <row r="92" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A92" s="4" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B92" s="4" t="s">
         <v>4</v>
@@ -50278,7 +50293,7 @@
     </row>
     <row r="93" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A93" s="7" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B93" s="8" t="s">
         <v>5</v>
@@ -50385,7 +50400,7 @@
     </row>
     <row r="94" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A94" s="12" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B94" s="4" t="s">
         <v>4</v>
@@ -50492,7 +50507,7 @@
     </row>
     <row r="95" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A95" s="12" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B95" s="4" t="s">
         <v>4</v>
@@ -50599,7 +50614,7 @@
     </row>
     <row r="96" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A96" s="12" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B96" s="4" t="s">
         <v>4</v>
@@ -50706,7 +50721,7 @@
     </row>
     <row r="97" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A97" s="4" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B97" s="4" t="s">
         <v>4</v>
@@ -50813,7 +50828,7 @@
     </row>
     <row r="98" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A98" s="4" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B98" s="4" t="s">
         <v>4</v>
@@ -50920,7 +50935,7 @@
     </row>
     <row r="99" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A99" s="28" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B99" s="28" t="s">
         <v>4</v>
@@ -51027,13 +51042,13 @@
     </row>
     <row r="100" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A100" s="4" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B100" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D100" s="2">
         <v>0</v>
@@ -51134,13 +51149,13 @@
     </row>
     <row r="101" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A101" s="4" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B101" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D101" s="2">
         <v>0</v>
@@ -51241,13 +51256,13 @@
     </row>
     <row r="102" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A102" s="4" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B102" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D102" s="2">
         <v>0</v>
@@ -51348,7 +51363,7 @@
     </row>
     <row r="103" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A103" s="7" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B103" s="8" t="s">
         <v>5</v>
@@ -51455,7 +51470,7 @@
     </row>
     <row r="104" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A104" s="28" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B104" s="28" t="s">
         <v>4</v>
@@ -51562,7 +51577,7 @@
     </row>
     <row r="105" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A105" s="12" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B105" s="4" t="s">
         <v>4</v>
@@ -51669,7 +51684,7 @@
     </row>
     <row r="106" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A106" s="12" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B106" s="4" t="s">
         <v>4</v>
@@ -51776,7 +51791,7 @@
     </row>
     <row r="107" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A107" s="12" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B107" s="4" t="s">
         <v>4</v>
@@ -51883,7 +51898,7 @@
     </row>
     <row r="108" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A108" s="28" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B108" s="28" t="s">
         <v>4</v>
@@ -51990,7 +52005,7 @@
     </row>
     <row r="109" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A109" s="7" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B109" s="8" t="s">
         <v>5</v>
@@ -52097,10 +52112,10 @@
     </row>
     <row r="110" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A110" s="4" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>8</v>
@@ -52204,10 +52219,10 @@
     </row>
     <row r="111" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A111" s="28" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B111" s="28" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>2</v>
@@ -52311,10 +52326,10 @@
     </row>
     <row r="112" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A112" s="4" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B112" s="12" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>2</v>
@@ -52418,10 +52433,10 @@
     </row>
     <row r="113" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A113" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B113" s="12" t="s">
         <v>89</v>
-      </c>
-      <c r="B113" s="12" t="s">
-        <v>93</v>
       </c>
       <c r="C113" s="1" t="s">
         <v>8</v>
@@ -52525,10 +52540,10 @@
     </row>
     <row r="114" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A114" s="4" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B114" s="12" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C114" s="1" t="s">
         <v>2</v>
@@ -52632,10 +52647,10 @@
     </row>
     <row r="115" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A115" s="28" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B115" s="28" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>2</v>
@@ -52739,10 +52754,10 @@
     </row>
     <row r="116" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A116" s="28" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B116" s="28" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>2</v>
@@ -52846,10 +52861,10 @@
     </row>
     <row r="117" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A117" s="4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B117" s="12" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>2</v>
@@ -52953,10 +52968,10 @@
     </row>
     <row r="118" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A118" s="4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B118" s="12" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>2</v>
@@ -53060,10 +53075,10 @@
     </row>
     <row r="119" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A119" s="28" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B119" s="28" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>2</v>
@@ -53167,10 +53182,10 @@
     </row>
     <row r="120" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A120" s="4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C120" s="1" t="s">
         <v>8</v>
@@ -53274,10 +53289,10 @@
     </row>
     <row r="121" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A121" s="28" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B121" s="28" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C121" s="1" t="s">
         <v>2</v>

</xml_diff>

<commit_message>
Financial statements formulas and welcome & country selection screens
Continuation of completing formulas in the financial statements for each model; pending verification of formulas at the end of the file and resolution of some formula-related doubts.

Welcome screen as the initial landing page for the tool.

Subsequent country selection screen to choose the implementation country.

Currently, only the Rwanda endpoint is included, as the tool development is based on this country.
</commit_message>
<xml_diff>
--- a/backend/financial-statements/financial-statements-template.xlsx
+++ b/backend/financial-statements/financial-statements-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8954da175e61d5af/Escritorio/IIT/NICCP-AI/backend/financial-statements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="492" documentId="10_ncr:20000_{4F2B366B-AA2F-4F18-863E-957538EF6F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD38011A-356D-4212-BBC1-C0084ABE4203}"/>
+  <xr:revisionPtr revIDLastSave="512" documentId="10_ncr:20000_{4F2B366B-AA2F-4F18-863E-957538EF6F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD6EC51C-8D29-4B98-9FC3-36DD2F6E7E4E}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="E-Cooking" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1779" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1930" uniqueCount="117">
   <si>
     <t>Units</t>
   </si>
@@ -192,9 +192,6 @@
   </si>
   <si>
     <t>Operating Cash Flow</t>
-  </si>
-  <si>
-    <t>Capex</t>
   </si>
   <si>
     <t>Investing Cash Flow</t>
@@ -390,6 +387,9 @@
   </si>
   <si>
     <t>- Cash movement</t>
+  </si>
+  <si>
+    <t>Capex for e-cooking + electrification plan</t>
   </si>
 </sst>
 </file>
@@ -1030,7 +1030,7 @@
   <sheetData>
     <row r="1" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>5</v>
@@ -3277,7 +3277,7 @@
     </row>
     <row r="22" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>4</v>
@@ -3491,7 +3491,7 @@
     </row>
     <row r="24" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>11</v>
@@ -4026,7 +4026,7 @@
     </row>
     <row r="29" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>4</v>
@@ -4240,7 +4240,7 @@
     </row>
     <row r="31" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>4</v>
@@ -4882,7 +4882,7 @@
     </row>
     <row r="37" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B37" s="8" t="s">
         <v>5</v>
@@ -5417,7 +5417,7 @@
     </row>
     <row r="42" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="29" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B42" s="30" t="s">
         <v>4</v>
@@ -6166,7 +6166,7 @@
     </row>
     <row r="49" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A49" s="29" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B49" s="30" t="s">
         <v>4</v>
@@ -6915,7 +6915,7 @@
     </row>
     <row r="56" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A56" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>4</v>
@@ -7450,7 +7450,7 @@
     </row>
     <row r="61" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A61" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B61" s="4" t="s">
         <v>4</v>
@@ -7985,7 +7985,7 @@
     </row>
     <row r="66" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A66" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B66" s="8" t="s">
         <v>5</v>
@@ -8092,7 +8092,7 @@
     </row>
     <row r="67" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A67" s="12" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>4</v>
@@ -8520,7 +8520,7 @@
     </row>
     <row r="71" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A71" s="4" t="s">
-        <v>51</v>
+        <v>116</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>4</v>
@@ -8627,7 +8627,7 @@
     </row>
     <row r="72" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A72" s="29" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B72" s="30" t="s">
         <v>4</v>
@@ -8734,7 +8734,7 @@
     </row>
     <row r="73" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A73" s="29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B73" s="30" t="s">
         <v>4</v>
@@ -8948,7 +8948,7 @@
     </row>
     <row r="75" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A75" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B75" s="4" t="s">
         <v>4</v>
@@ -9055,7 +9055,7 @@
     </row>
     <row r="76" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A76" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B76" s="4" t="s">
         <v>4</v>
@@ -9162,7 +9162,7 @@
     </row>
     <row r="77" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A77" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B77" s="4" t="s">
         <v>4</v>
@@ -9269,7 +9269,7 @@
     </row>
     <row r="78" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A78" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B78" s="4" t="s">
         <v>4</v>
@@ -9376,7 +9376,7 @@
     </row>
     <row r="79" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A79" s="12" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B79" s="4" t="s">
         <v>4</v>
@@ -9483,7 +9483,7 @@
     </row>
     <row r="80" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A80" s="29" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B80" s="30" t="s">
         <v>4</v>
@@ -9590,7 +9590,7 @@
     </row>
     <row r="81" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A81" s="29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B81" s="30" t="s">
         <v>4</v>
@@ -9697,7 +9697,7 @@
     </row>
     <row r="82" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A82" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B82" s="4" t="s">
         <v>4</v>
@@ -9804,7 +9804,7 @@
     </row>
     <row r="83" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A83" s="12" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B83" s="4" t="s">
         <v>4</v>
@@ -9911,7 +9911,7 @@
     </row>
     <row r="84" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A84" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B84" s="4" t="s">
         <v>4</v>
@@ -10018,7 +10018,7 @@
     </row>
     <row r="85" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A85" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B85" s="8" t="s">
         <v>5</v>
@@ -10125,7 +10125,7 @@
     </row>
     <row r="86" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A86" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B86" s="4" t="s">
         <v>4</v>
@@ -10232,7 +10232,7 @@
     </row>
     <row r="87" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A87" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>11</v>
@@ -10339,7 +10339,7 @@
     </row>
     <row r="88" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A88" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B88" s="4" t="s">
         <v>4</v>
@@ -10446,7 +10446,7 @@
     </row>
     <row r="89" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A89" s="12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>4</v>
@@ -10553,7 +10553,7 @@
     </row>
     <row r="90" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A90" s="12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B90" s="4" t="s">
         <v>4</v>
@@ -10660,7 +10660,7 @@
     </row>
     <row r="91" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A91" s="12" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B91" s="4" t="s">
         <v>4</v>
@@ -10767,7 +10767,7 @@
     </row>
     <row r="92" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A92" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B92" s="4" t="s">
         <v>4</v>
@@ -10874,7 +10874,7 @@
     </row>
     <row r="93" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A93" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B93" s="8" t="s">
         <v>5</v>
@@ -10981,7 +10981,7 @@
     </row>
     <row r="94" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A94" s="12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B94" s="4" t="s">
         <v>4</v>
@@ -11088,7 +11088,7 @@
     </row>
     <row r="95" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A95" s="12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B95" s="4" t="s">
         <v>4</v>
@@ -11195,7 +11195,7 @@
     </row>
     <row r="96" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A96" s="12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B96" s="4" t="s">
         <v>4</v>
@@ -11302,7 +11302,7 @@
     </row>
     <row r="97" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A97" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B97" s="4" t="s">
         <v>4</v>
@@ -11409,7 +11409,7 @@
     </row>
     <row r="98" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A98" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B98" s="4" t="s">
         <v>4</v>
@@ -11516,7 +11516,7 @@
     </row>
     <row r="99" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A99" s="28" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B99" s="28" t="s">
         <v>4</v>
@@ -11623,13 +11623,13 @@
     </row>
     <row r="100" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A100" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B100" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D100" s="2">
         <v>0</v>
@@ -11730,13 +11730,13 @@
     </row>
     <row r="101" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A101" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B101" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D101" s="2">
         <v>0</v>
@@ -11837,13 +11837,13 @@
     </row>
     <row r="102" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A102" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C102" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="B102" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C102" s="1" t="s">
-        <v>80</v>
       </c>
       <c r="D102" s="2">
         <v>0</v>
@@ -11944,7 +11944,7 @@
     </row>
     <row r="103" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A103" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B103" s="8" t="s">
         <v>5</v>
@@ -12051,7 +12051,7 @@
     </row>
     <row r="104" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A104" s="28" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B104" s="28" t="s">
         <v>4</v>
@@ -12158,7 +12158,7 @@
     </row>
     <row r="105" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A105" s="12" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B105" s="4" t="s">
         <v>4</v>
@@ -12169,103 +12169,103 @@
       <c r="D105" s="2">
         <v>0</v>
       </c>
-      <c r="E105" s="2">
-        <v>0</v>
-      </c>
-      <c r="F105" s="2">
-        <v>0</v>
-      </c>
-      <c r="G105" s="2">
-        <v>0</v>
-      </c>
-      <c r="H105" s="2">
-        <v>0</v>
-      </c>
-      <c r="I105" s="2">
-        <v>0</v>
-      </c>
-      <c r="J105" s="2">
-        <v>0</v>
-      </c>
-      <c r="K105" s="2">
-        <v>0</v>
-      </c>
-      <c r="L105" s="2">
-        <v>0</v>
-      </c>
-      <c r="M105" s="2">
-        <v>0</v>
-      </c>
-      <c r="N105" s="2">
-        <v>0</v>
-      </c>
-      <c r="O105" s="2">
-        <v>0</v>
-      </c>
-      <c r="P105" s="2">
-        <v>0</v>
-      </c>
-      <c r="Q105" s="2">
-        <v>0</v>
-      </c>
-      <c r="R105" s="2">
-        <v>0</v>
-      </c>
-      <c r="S105" s="2">
-        <v>0</v>
-      </c>
-      <c r="T105" s="2">
-        <v>0</v>
-      </c>
-      <c r="U105" s="2">
-        <v>0</v>
-      </c>
-      <c r="V105" s="2">
-        <v>0</v>
-      </c>
-      <c r="W105" s="2">
-        <v>0</v>
-      </c>
-      <c r="X105" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y105" s="2">
-        <v>0</v>
-      </c>
-      <c r="Z105" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA105" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB105" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC105" s="2">
-        <v>0</v>
-      </c>
-      <c r="AD105" s="2">
-        <v>0</v>
-      </c>
-      <c r="AE105" s="2">
-        <v>0</v>
-      </c>
-      <c r="AF105" s="2">
-        <v>0</v>
-      </c>
-      <c r="AG105" s="2">
-        <v>0</v>
-      </c>
-      <c r="AH105" s="2">
-        <v>0</v>
-      </c>
-      <c r="AI105" s="2">
-        <v>0</v>
+      <c r="E105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="F105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="G105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="H105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="I105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="J105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="K105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="L105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="M105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="N105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="O105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="P105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="R105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="S105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="T105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="U105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="V105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="W105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="X105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="Y105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="Z105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AA105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AB105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AC105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AD105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AE105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AF105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AG105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AH105" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AI105" s="27" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="106" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A106" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B106" s="4" t="s">
         <v>4</v>
@@ -12276,103 +12276,103 @@
       <c r="D106" s="2">
         <v>0</v>
       </c>
-      <c r="E106" s="2">
-        <v>0</v>
-      </c>
-      <c r="F106" s="2">
-        <v>0</v>
-      </c>
-      <c r="G106" s="2">
-        <v>0</v>
-      </c>
-      <c r="H106" s="2">
-        <v>0</v>
-      </c>
-      <c r="I106" s="2">
-        <v>0</v>
-      </c>
-      <c r="J106" s="2">
-        <v>0</v>
-      </c>
-      <c r="K106" s="2">
-        <v>0</v>
-      </c>
-      <c r="L106" s="2">
-        <v>0</v>
-      </c>
-      <c r="M106" s="2">
-        <v>0</v>
-      </c>
-      <c r="N106" s="2">
-        <v>0</v>
-      </c>
-      <c r="O106" s="2">
-        <v>0</v>
-      </c>
-      <c r="P106" s="2">
-        <v>0</v>
-      </c>
-      <c r="Q106" s="2">
-        <v>0</v>
-      </c>
-      <c r="R106" s="2">
-        <v>0</v>
-      </c>
-      <c r="S106" s="2">
-        <v>0</v>
-      </c>
-      <c r="T106" s="2">
-        <v>0</v>
-      </c>
-      <c r="U106" s="2">
-        <v>0</v>
-      </c>
-      <c r="V106" s="2">
-        <v>0</v>
-      </c>
-      <c r="W106" s="2">
-        <v>0</v>
-      </c>
-      <c r="X106" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y106" s="2">
-        <v>0</v>
-      </c>
-      <c r="Z106" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA106" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB106" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC106" s="2">
-        <v>0</v>
-      </c>
-      <c r="AD106" s="2">
-        <v>0</v>
-      </c>
-      <c r="AE106" s="2">
-        <v>0</v>
-      </c>
-      <c r="AF106" s="2">
-        <v>0</v>
-      </c>
-      <c r="AG106" s="2">
-        <v>0</v>
-      </c>
-      <c r="AH106" s="2">
-        <v>0</v>
-      </c>
-      <c r="AI106" s="2">
+      <c r="E106" s="27">
+        <v>0</v>
+      </c>
+      <c r="F106" s="27">
+        <v>0</v>
+      </c>
+      <c r="G106" s="27">
+        <v>0</v>
+      </c>
+      <c r="H106" s="27">
+        <v>0</v>
+      </c>
+      <c r="I106" s="27">
+        <v>0</v>
+      </c>
+      <c r="J106" s="27">
+        <v>0</v>
+      </c>
+      <c r="K106" s="27">
+        <v>0</v>
+      </c>
+      <c r="L106" s="27">
+        <v>0</v>
+      </c>
+      <c r="M106" s="27">
+        <v>0</v>
+      </c>
+      <c r="N106" s="27">
+        <v>0</v>
+      </c>
+      <c r="O106" s="27">
+        <v>0</v>
+      </c>
+      <c r="P106" s="27">
+        <v>0</v>
+      </c>
+      <c r="Q106" s="27">
+        <v>0</v>
+      </c>
+      <c r="R106" s="27">
+        <v>0</v>
+      </c>
+      <c r="S106" s="27">
+        <v>0</v>
+      </c>
+      <c r="T106" s="27">
+        <v>0</v>
+      </c>
+      <c r="U106" s="27">
+        <v>0</v>
+      </c>
+      <c r="V106" s="27">
+        <v>0</v>
+      </c>
+      <c r="W106" s="27">
+        <v>0</v>
+      </c>
+      <c r="X106" s="27">
+        <v>0</v>
+      </c>
+      <c r="Y106" s="27">
+        <v>0</v>
+      </c>
+      <c r="Z106" s="27">
+        <v>0</v>
+      </c>
+      <c r="AA106" s="27">
+        <v>0</v>
+      </c>
+      <c r="AB106" s="27">
+        <v>0</v>
+      </c>
+      <c r="AC106" s="27">
+        <v>0</v>
+      </c>
+      <c r="AD106" s="27">
+        <v>0</v>
+      </c>
+      <c r="AE106" s="27">
+        <v>0</v>
+      </c>
+      <c r="AF106" s="27">
+        <v>0</v>
+      </c>
+      <c r="AG106" s="27">
+        <v>0</v>
+      </c>
+      <c r="AH106" s="27">
+        <v>0</v>
+      </c>
+      <c r="AI106" s="27">
         <v>0</v>
       </c>
     </row>
     <row r="107" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A107" s="12" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B107" s="4" t="s">
         <v>4</v>
@@ -12479,7 +12479,7 @@
     </row>
     <row r="108" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A108" s="28" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B108" s="28" t="s">
         <v>4</v>
@@ -12586,7 +12586,7 @@
     </row>
     <row r="109" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A109" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B109" s="8" t="s">
         <v>5</v>
@@ -12693,10 +12693,10 @@
     </row>
     <row r="110" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A110" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B110" s="4" t="s">
         <v>85</v>
-      </c>
-      <c r="B110" s="4" t="s">
-        <v>86</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>8</v>
@@ -12800,10 +12800,10 @@
     </row>
     <row r="111" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A111" s="28" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B111" s="28" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>2</v>
@@ -12907,10 +12907,10 @@
     </row>
     <row r="112" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A112" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B112" s="12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>2</v>
@@ -12921,106 +12921,106 @@
       <c r="E112" s="2">
         <v>0</v>
       </c>
-      <c r="F112" s="2">
-        <v>0</v>
-      </c>
-      <c r="G112" s="2">
-        <v>0</v>
-      </c>
-      <c r="H112" s="2">
-        <v>0</v>
-      </c>
-      <c r="I112" s="2">
-        <v>0</v>
-      </c>
-      <c r="J112" s="2">
-        <v>0</v>
-      </c>
-      <c r="K112" s="2">
-        <v>0</v>
-      </c>
-      <c r="L112" s="2">
-        <v>0</v>
-      </c>
-      <c r="M112" s="2">
-        <v>0</v>
-      </c>
-      <c r="N112" s="2">
-        <v>0</v>
-      </c>
-      <c r="O112" s="2">
-        <v>0</v>
-      </c>
-      <c r="P112" s="2">
-        <v>0</v>
-      </c>
-      <c r="Q112" s="2">
-        <v>0</v>
-      </c>
-      <c r="R112" s="2">
-        <v>0</v>
-      </c>
-      <c r="S112" s="2">
-        <v>0</v>
-      </c>
-      <c r="T112" s="2">
-        <v>0</v>
-      </c>
-      <c r="U112" s="2">
-        <v>0</v>
-      </c>
-      <c r="V112" s="2">
-        <v>0</v>
-      </c>
-      <c r="W112" s="2">
-        <v>0</v>
-      </c>
-      <c r="X112" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y112" s="2">
-        <v>0</v>
-      </c>
-      <c r="Z112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AD112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AE112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AF112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AG112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AH112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AI112" s="2">
-        <v>0</v>
+      <c r="F112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="G112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="H112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="I112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="J112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="K112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="L112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="M112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="N112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="O112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="P112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="R112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="S112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="T112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="U112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="V112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="W112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="X112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="Y112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="Z112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AA112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AB112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AC112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AD112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AE112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AF112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AG112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AH112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AI112" s="27" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="113" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A113" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B113" s="12" t="s">
         <v>89</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D113" s="2">
         <v>0</v>
@@ -13121,13 +13121,13 @@
     </row>
     <row r="114" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A114" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B114" s="12" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D114" s="2">
         <v>0</v>
@@ -13228,10 +13228,10 @@
     </row>
     <row r="115" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A115" s="28" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B115" s="28" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>2</v>
@@ -13335,10 +13335,10 @@
     </row>
     <row r="116" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A116" s="28" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B116" s="28" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>2</v>
@@ -13442,10 +13442,10 @@
     </row>
     <row r="117" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A117" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B117" s="12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>2</v>
@@ -13549,10 +13549,10 @@
     </row>
     <row r="118" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A118" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B118" s="12" t="s">
         <v>92</v>
-      </c>
-      <c r="B118" s="12" t="s">
-        <v>93</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>2</v>
@@ -13656,10 +13656,10 @@
     </row>
     <row r="119" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A119" s="28" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B119" s="28" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>2</v>
@@ -13763,10 +13763,10 @@
     </row>
     <row r="120" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A120" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C120" s="1" t="s">
         <v>8</v>
@@ -13870,10 +13870,10 @@
     </row>
     <row r="121" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A121" s="28" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B121" s="28" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C121" s="1" t="s">
         <v>2</v>
@@ -13991,7 +13991,7 @@
   <sheetData>
     <row r="1" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>5</v>
@@ -16238,7 +16238,7 @@
     </row>
     <row r="22" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>4</v>
@@ -16452,7 +16452,7 @@
     </row>
     <row r="24" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>11</v>
@@ -16987,7 +16987,7 @@
     </row>
     <row r="29" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>4</v>
@@ -17201,7 +17201,7 @@
     </row>
     <row r="31" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>4</v>
@@ -17843,7 +17843,7 @@
     </row>
     <row r="37" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B37" s="8" t="s">
         <v>5</v>
@@ -18378,7 +18378,7 @@
     </row>
     <row r="42" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="29" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B42" s="30" t="s">
         <v>4</v>
@@ -19127,7 +19127,7 @@
     </row>
     <row r="49" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A49" s="29" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B49" s="30" t="s">
         <v>4</v>
@@ -19876,7 +19876,7 @@
     </row>
     <row r="56" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A56" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>4</v>
@@ -20411,7 +20411,7 @@
     </row>
     <row r="61" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A61" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B61" s="4" t="s">
         <v>4</v>
@@ -20946,7 +20946,7 @@
     </row>
     <row r="66" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A66" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B66" s="8" t="s">
         <v>5</v>
@@ -21053,7 +21053,7 @@
     </row>
     <row r="67" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A67" s="12" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>4</v>
@@ -21481,7 +21481,7 @@
     </row>
     <row r="71" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A71" s="4" t="s">
-        <v>51</v>
+        <v>116</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>4</v>
@@ -21588,7 +21588,7 @@
     </row>
     <row r="72" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A72" s="29" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B72" s="30" t="s">
         <v>4</v>
@@ -21695,7 +21695,7 @@
     </row>
     <row r="73" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A73" s="29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B73" s="30" t="s">
         <v>4</v>
@@ -21909,7 +21909,7 @@
     </row>
     <row r="75" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A75" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B75" s="4" t="s">
         <v>4</v>
@@ -22016,7 +22016,7 @@
     </row>
     <row r="76" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A76" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B76" s="4" t="s">
         <v>4</v>
@@ -22123,7 +22123,7 @@
     </row>
     <row r="77" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A77" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B77" s="4" t="s">
         <v>4</v>
@@ -22230,7 +22230,7 @@
     </row>
     <row r="78" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A78" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B78" s="4" t="s">
         <v>4</v>
@@ -22337,7 +22337,7 @@
     </row>
     <row r="79" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A79" s="12" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B79" s="4" t="s">
         <v>4</v>
@@ -22444,7 +22444,7 @@
     </row>
     <row r="80" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A80" s="29" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B80" s="30" t="s">
         <v>4</v>
@@ -22551,7 +22551,7 @@
     </row>
     <row r="81" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A81" s="29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B81" s="30" t="s">
         <v>4</v>
@@ -22658,7 +22658,7 @@
     </row>
     <row r="82" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A82" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B82" s="4" t="s">
         <v>4</v>
@@ -22765,7 +22765,7 @@
     </row>
     <row r="83" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A83" s="12" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B83" s="4" t="s">
         <v>4</v>
@@ -22872,7 +22872,7 @@
     </row>
     <row r="84" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A84" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B84" s="4" t="s">
         <v>4</v>
@@ -22979,7 +22979,7 @@
     </row>
     <row r="85" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A85" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B85" s="8" t="s">
         <v>5</v>
@@ -23086,7 +23086,7 @@
     </row>
     <row r="86" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A86" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B86" s="4" t="s">
         <v>4</v>
@@ -23193,7 +23193,7 @@
     </row>
     <row r="87" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A87" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>11</v>
@@ -23300,7 +23300,7 @@
     </row>
     <row r="88" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A88" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B88" s="4" t="s">
         <v>4</v>
@@ -23407,7 +23407,7 @@
     </row>
     <row r="89" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A89" s="12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>4</v>
@@ -23514,7 +23514,7 @@
     </row>
     <row r="90" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A90" s="12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B90" s="4" t="s">
         <v>4</v>
@@ -23621,7 +23621,7 @@
     </row>
     <row r="91" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A91" s="12" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B91" s="4" t="s">
         <v>4</v>
@@ -23728,7 +23728,7 @@
     </row>
     <row r="92" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A92" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B92" s="4" t="s">
         <v>4</v>
@@ -23835,7 +23835,7 @@
     </row>
     <row r="93" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A93" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B93" s="8" t="s">
         <v>5</v>
@@ -23942,7 +23942,7 @@
     </row>
     <row r="94" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A94" s="12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B94" s="4" t="s">
         <v>4</v>
@@ -24049,7 +24049,7 @@
     </row>
     <row r="95" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A95" s="12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B95" s="4" t="s">
         <v>4</v>
@@ -24156,7 +24156,7 @@
     </row>
     <row r="96" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A96" s="12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B96" s="4" t="s">
         <v>4</v>
@@ -24263,7 +24263,7 @@
     </row>
     <row r="97" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A97" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B97" s="4" t="s">
         <v>4</v>
@@ -24370,7 +24370,7 @@
     </row>
     <row r="98" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A98" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B98" s="4" t="s">
         <v>4</v>
@@ -24477,7 +24477,7 @@
     </row>
     <row r="99" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A99" s="28" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B99" s="28" t="s">
         <v>4</v>
@@ -24584,13 +24584,13 @@
     </row>
     <row r="100" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A100" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B100" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D100" s="2">
         <v>0</v>
@@ -24691,13 +24691,13 @@
     </row>
     <row r="101" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A101" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B101" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D101" s="2">
         <v>0</v>
@@ -24798,13 +24798,13 @@
     </row>
     <row r="102" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A102" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C102" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="B102" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C102" s="1" t="s">
-        <v>80</v>
       </c>
       <c r="D102" s="2">
         <v>0</v>
@@ -24905,7 +24905,7 @@
     </row>
     <row r="103" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A103" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B103" s="8" t="s">
         <v>5</v>
@@ -25012,7 +25012,7 @@
     </row>
     <row r="104" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A104" s="28" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B104" s="28" t="s">
         <v>4</v>
@@ -25119,7 +25119,7 @@
     </row>
     <row r="105" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A105" s="12" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B105" s="4" t="s">
         <v>4</v>
@@ -25226,7 +25226,7 @@
     </row>
     <row r="106" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A106" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B106" s="4" t="s">
         <v>4</v>
@@ -25333,7 +25333,7 @@
     </row>
     <row r="107" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A107" s="12" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B107" s="4" t="s">
         <v>4</v>
@@ -25440,7 +25440,7 @@
     </row>
     <row r="108" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A108" s="28" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B108" s="28" t="s">
         <v>4</v>
@@ -25547,7 +25547,7 @@
     </row>
     <row r="109" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A109" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B109" s="8" t="s">
         <v>5</v>
@@ -25654,10 +25654,10 @@
     </row>
     <row r="110" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A110" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B110" s="4" t="s">
         <v>85</v>
-      </c>
-      <c r="B110" s="4" t="s">
-        <v>86</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>8</v>
@@ -25761,10 +25761,10 @@
     </row>
     <row r="111" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A111" s="28" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B111" s="28" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>2</v>
@@ -25868,10 +25868,10 @@
     </row>
     <row r="112" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A112" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B112" s="12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>2</v>
@@ -25882,106 +25882,106 @@
       <c r="E112" s="2">
         <v>0</v>
       </c>
-      <c r="F112" s="2">
-        <v>0</v>
-      </c>
-      <c r="G112" s="2">
-        <v>0</v>
-      </c>
-      <c r="H112" s="2">
-        <v>0</v>
-      </c>
-      <c r="I112" s="2">
-        <v>0</v>
-      </c>
-      <c r="J112" s="2">
-        <v>0</v>
-      </c>
-      <c r="K112" s="2">
-        <v>0</v>
-      </c>
-      <c r="L112" s="2">
-        <v>0</v>
-      </c>
-      <c r="M112" s="2">
-        <v>0</v>
-      </c>
-      <c r="N112" s="2">
-        <v>0</v>
-      </c>
-      <c r="O112" s="2">
-        <v>0</v>
-      </c>
-      <c r="P112" s="2">
-        <v>0</v>
-      </c>
-      <c r="Q112" s="2">
-        <v>0</v>
-      </c>
-      <c r="R112" s="2">
-        <v>0</v>
-      </c>
-      <c r="S112" s="2">
-        <v>0</v>
-      </c>
-      <c r="T112" s="2">
-        <v>0</v>
-      </c>
-      <c r="U112" s="2">
-        <v>0</v>
-      </c>
-      <c r="V112" s="2">
-        <v>0</v>
-      </c>
-      <c r="W112" s="2">
-        <v>0</v>
-      </c>
-      <c r="X112" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y112" s="2">
-        <v>0</v>
-      </c>
-      <c r="Z112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AD112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AE112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AF112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AG112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AH112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AI112" s="2">
-        <v>0</v>
+      <c r="F112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="G112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="H112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="I112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="J112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="K112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="L112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="M112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="N112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="O112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="P112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="R112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="S112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="T112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="U112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="V112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="W112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="X112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="Y112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="Z112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AA112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AB112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AC112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AD112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AE112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AF112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AG112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AH112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AI112" s="27" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="113" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A113" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B113" s="12" t="s">
         <v>89</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D113" s="2">
         <v>0</v>
@@ -26082,13 +26082,13 @@
     </row>
     <row r="114" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A114" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B114" s="12" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D114" s="2">
         <v>0</v>
@@ -26189,10 +26189,10 @@
     </row>
     <row r="115" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A115" s="28" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B115" s="28" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>2</v>
@@ -26296,10 +26296,10 @@
     </row>
     <row r="116" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A116" s="28" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B116" s="28" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>2</v>
@@ -26403,10 +26403,10 @@
     </row>
     <row r="117" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A117" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B117" s="12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>2</v>
@@ -26510,10 +26510,10 @@
     </row>
     <row r="118" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A118" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B118" s="12" t="s">
         <v>92</v>
-      </c>
-      <c r="B118" s="12" t="s">
-        <v>93</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>2</v>
@@ -26617,10 +26617,10 @@
     </row>
     <row r="119" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A119" s="28" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B119" s="28" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>2</v>
@@ -26724,10 +26724,10 @@
     </row>
     <row r="120" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A120" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C120" s="1" t="s">
         <v>8</v>
@@ -26831,10 +26831,10 @@
     </row>
     <row r="121" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A121" s="28" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B121" s="28" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C121" s="1" t="s">
         <v>2</v>
@@ -26952,7 +26952,7 @@
   <sheetData>
     <row r="1" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>5</v>
@@ -29199,7 +29199,7 @@
     </row>
     <row r="22" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>4</v>
@@ -29413,7 +29413,7 @@
     </row>
     <row r="24" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>11</v>
@@ -29948,7 +29948,7 @@
     </row>
     <row r="29" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>4</v>
@@ -30162,7 +30162,7 @@
     </row>
     <row r="31" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>4</v>
@@ -30804,7 +30804,7 @@
     </row>
     <row r="37" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B37" s="8" t="s">
         <v>5</v>
@@ -31339,7 +31339,7 @@
     </row>
     <row r="42" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="29" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B42" s="30" t="s">
         <v>4</v>
@@ -32088,7 +32088,7 @@
     </row>
     <row r="49" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A49" s="29" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B49" s="30" t="s">
         <v>4</v>
@@ -32837,7 +32837,7 @@
     </row>
     <row r="56" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A56" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>4</v>
@@ -33372,7 +33372,7 @@
     </row>
     <row r="61" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A61" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B61" s="4" t="s">
         <v>4</v>
@@ -33907,7 +33907,7 @@
     </row>
     <row r="66" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A66" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B66" s="8" t="s">
         <v>5</v>
@@ -34014,7 +34014,7 @@
     </row>
     <row r="67" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A67" s="12" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>4</v>
@@ -34442,7 +34442,7 @@
     </row>
     <row r="71" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A71" s="4" t="s">
-        <v>51</v>
+        <v>116</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>4</v>
@@ -34549,7 +34549,7 @@
     </row>
     <row r="72" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A72" s="29" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B72" s="30" t="s">
         <v>4</v>
@@ -34656,7 +34656,7 @@
     </row>
     <row r="73" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A73" s="29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B73" s="30" t="s">
         <v>4</v>
@@ -34870,7 +34870,7 @@
     </row>
     <row r="75" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A75" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B75" s="4" t="s">
         <v>4</v>
@@ -34977,7 +34977,7 @@
     </row>
     <row r="76" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A76" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B76" s="4" t="s">
         <v>4</v>
@@ -35084,7 +35084,7 @@
     </row>
     <row r="77" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A77" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B77" s="4" t="s">
         <v>4</v>
@@ -35191,7 +35191,7 @@
     </row>
     <row r="78" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A78" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B78" s="4" t="s">
         <v>4</v>
@@ -35298,7 +35298,7 @@
     </row>
     <row r="79" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A79" s="12" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B79" s="4" t="s">
         <v>4</v>
@@ -35405,7 +35405,7 @@
     </row>
     <row r="80" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A80" s="29" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B80" s="30" t="s">
         <v>4</v>
@@ -35512,7 +35512,7 @@
     </row>
     <row r="81" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A81" s="29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B81" s="30" t="s">
         <v>4</v>
@@ -35619,7 +35619,7 @@
     </row>
     <row r="82" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A82" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B82" s="4" t="s">
         <v>4</v>
@@ -35726,7 +35726,7 @@
     </row>
     <row r="83" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A83" s="12" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B83" s="4" t="s">
         <v>4</v>
@@ -35833,7 +35833,7 @@
     </row>
     <row r="84" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A84" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B84" s="4" t="s">
         <v>4</v>
@@ -35940,7 +35940,7 @@
     </row>
     <row r="85" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A85" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B85" s="8" t="s">
         <v>5</v>
@@ -36047,7 +36047,7 @@
     </row>
     <row r="86" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A86" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B86" s="4" t="s">
         <v>4</v>
@@ -36154,7 +36154,7 @@
     </row>
     <row r="87" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A87" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>11</v>
@@ -36261,7 +36261,7 @@
     </row>
     <row r="88" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A88" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B88" s="4" t="s">
         <v>4</v>
@@ -36368,7 +36368,7 @@
     </row>
     <row r="89" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A89" s="12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>4</v>
@@ -36475,7 +36475,7 @@
     </row>
     <row r="90" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A90" s="12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B90" s="4" t="s">
         <v>4</v>
@@ -36582,7 +36582,7 @@
     </row>
     <row r="91" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A91" s="12" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B91" s="4" t="s">
         <v>4</v>
@@ -36689,7 +36689,7 @@
     </row>
     <row r="92" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A92" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B92" s="4" t="s">
         <v>4</v>
@@ -36796,7 +36796,7 @@
     </row>
     <row r="93" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A93" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B93" s="8" t="s">
         <v>5</v>
@@ -36903,7 +36903,7 @@
     </row>
     <row r="94" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A94" s="12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B94" s="4" t="s">
         <v>4</v>
@@ -37010,7 +37010,7 @@
     </row>
     <row r="95" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A95" s="12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B95" s="4" t="s">
         <v>4</v>
@@ -37117,7 +37117,7 @@
     </row>
     <row r="96" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A96" s="12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B96" s="4" t="s">
         <v>4</v>
@@ -37224,7 +37224,7 @@
     </row>
     <row r="97" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A97" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B97" s="4" t="s">
         <v>4</v>
@@ -37331,7 +37331,7 @@
     </row>
     <row r="98" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A98" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B98" s="4" t="s">
         <v>4</v>
@@ -37438,7 +37438,7 @@
     </row>
     <row r="99" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A99" s="28" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B99" s="28" t="s">
         <v>4</v>
@@ -37545,13 +37545,13 @@
     </row>
     <row r="100" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A100" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B100" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D100" s="2">
         <v>0</v>
@@ -37652,13 +37652,13 @@
     </row>
     <row r="101" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A101" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B101" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D101" s="2">
         <v>0</v>
@@ -37759,13 +37759,13 @@
     </row>
     <row r="102" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A102" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C102" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="B102" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C102" s="1" t="s">
-        <v>80</v>
       </c>
       <c r="D102" s="2">
         <v>0</v>
@@ -37866,7 +37866,7 @@
     </row>
     <row r="103" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A103" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B103" s="8" t="s">
         <v>5</v>
@@ -37973,7 +37973,7 @@
     </row>
     <row r="104" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A104" s="28" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B104" s="28" t="s">
         <v>4</v>
@@ -38080,7 +38080,7 @@
     </row>
     <row r="105" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A105" s="12" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B105" s="4" t="s">
         <v>4</v>
@@ -38187,7 +38187,7 @@
     </row>
     <row r="106" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A106" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B106" s="4" t="s">
         <v>4</v>
@@ -38294,7 +38294,7 @@
     </row>
     <row r="107" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A107" s="12" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B107" s="4" t="s">
         <v>4</v>
@@ -38401,7 +38401,7 @@
     </row>
     <row r="108" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A108" s="28" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B108" s="28" t="s">
         <v>4</v>
@@ -38508,7 +38508,7 @@
     </row>
     <row r="109" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A109" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B109" s="8" t="s">
         <v>5</v>
@@ -38615,10 +38615,10 @@
     </row>
     <row r="110" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A110" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B110" s="4" t="s">
         <v>85</v>
-      </c>
-      <c r="B110" s="4" t="s">
-        <v>86</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>8</v>
@@ -38722,10 +38722,10 @@
     </row>
     <row r="111" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A111" s="28" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B111" s="28" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>2</v>
@@ -38829,10 +38829,10 @@
     </row>
     <row r="112" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A112" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B112" s="12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>2</v>
@@ -38843,106 +38843,106 @@
       <c r="E112" s="2">
         <v>0</v>
       </c>
-      <c r="F112" s="2">
-        <v>0</v>
-      </c>
-      <c r="G112" s="2">
-        <v>0</v>
-      </c>
-      <c r="H112" s="2">
-        <v>0</v>
-      </c>
-      <c r="I112" s="2">
-        <v>0</v>
-      </c>
-      <c r="J112" s="2">
-        <v>0</v>
-      </c>
-      <c r="K112" s="2">
-        <v>0</v>
-      </c>
-      <c r="L112" s="2">
-        <v>0</v>
-      </c>
-      <c r="M112" s="2">
-        <v>0</v>
-      </c>
-      <c r="N112" s="2">
-        <v>0</v>
-      </c>
-      <c r="O112" s="2">
-        <v>0</v>
-      </c>
-      <c r="P112" s="2">
-        <v>0</v>
-      </c>
-      <c r="Q112" s="2">
-        <v>0</v>
-      </c>
-      <c r="R112" s="2">
-        <v>0</v>
-      </c>
-      <c r="S112" s="2">
-        <v>0</v>
-      </c>
-      <c r="T112" s="2">
-        <v>0</v>
-      </c>
-      <c r="U112" s="2">
-        <v>0</v>
-      </c>
-      <c r="V112" s="2">
-        <v>0</v>
-      </c>
-      <c r="W112" s="2">
-        <v>0</v>
-      </c>
-      <c r="X112" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y112" s="2">
-        <v>0</v>
-      </c>
-      <c r="Z112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AD112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AE112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AF112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AG112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AH112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AI112" s="2">
-        <v>0</v>
+      <c r="F112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="G112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="H112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="I112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="J112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="K112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="L112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="M112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="N112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="O112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="P112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="R112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="S112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="T112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="U112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="V112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="W112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="X112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="Y112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="Z112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AA112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AB112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AC112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AD112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AE112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AF112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AG112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AH112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AI112" s="27" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="113" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A113" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B113" s="12" t="s">
         <v>89</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D113" s="2">
         <v>0</v>
@@ -39043,13 +39043,13 @@
     </row>
     <row r="114" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A114" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B114" s="12" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D114" s="2">
         <v>0</v>
@@ -39150,10 +39150,10 @@
     </row>
     <row r="115" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A115" s="28" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B115" s="28" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>2</v>
@@ -39257,10 +39257,10 @@
     </row>
     <row r="116" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A116" s="28" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B116" s="28" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>2</v>
@@ -39364,10 +39364,10 @@
     </row>
     <row r="117" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A117" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B117" s="12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>2</v>
@@ -39471,10 +39471,10 @@
     </row>
     <row r="118" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A118" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B118" s="12" t="s">
         <v>92</v>
-      </c>
-      <c r="B118" s="12" t="s">
-        <v>93</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>2</v>
@@ -39578,10 +39578,10 @@
     </row>
     <row r="119" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A119" s="28" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B119" s="28" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>2</v>
@@ -39685,10 +39685,10 @@
     </row>
     <row r="120" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A120" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C120" s="1" t="s">
         <v>8</v>
@@ -39792,10 +39792,10 @@
     </row>
     <row r="121" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A121" s="28" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B121" s="28" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C121" s="1" t="s">
         <v>2</v>
@@ -39899,7 +39899,7 @@
     </row>
     <row r="122" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A122" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B122" s="8" t="s">
         <v>5</v>
@@ -40006,7 +40006,7 @@
     </row>
     <row r="123" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A123" s="12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B123" s="4" t="s">
         <v>4</v>
@@ -40113,7 +40113,7 @@
     </row>
     <row r="124" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A124" s="12" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B124" s="4" t="s">
         <v>4</v>
@@ -40220,13 +40220,13 @@
     </row>
     <row r="125" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A125" s="12" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B125" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D125" s="2">
         <v>0</v>
@@ -40327,7 +40327,7 @@
     </row>
     <row r="126" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A126" s="23" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B126" s="24" t="s">
         <v>4</v>
@@ -40449,7 +40449,7 @@
   <sheetData>
     <row r="1" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>5</v>
@@ -42696,7 +42696,7 @@
     </row>
     <row r="22" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>4</v>
@@ -42910,7 +42910,7 @@
     </row>
     <row r="24" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>11</v>
@@ -43445,7 +43445,7 @@
     </row>
     <row r="29" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>4</v>
@@ -43659,7 +43659,7 @@
     </row>
     <row r="31" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>4</v>
@@ -44301,7 +44301,7 @@
     </row>
     <row r="37" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B37" s="8" t="s">
         <v>5</v>
@@ -44836,7 +44836,7 @@
     </row>
     <row r="42" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="29" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B42" s="30" t="s">
         <v>4</v>
@@ -45585,7 +45585,7 @@
     </row>
     <row r="49" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A49" s="29" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B49" s="30" t="s">
         <v>4</v>
@@ -46334,7 +46334,7 @@
     </row>
     <row r="56" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A56" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>4</v>
@@ -46869,7 +46869,7 @@
     </row>
     <row r="61" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A61" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B61" s="4" t="s">
         <v>4</v>
@@ -47404,7 +47404,7 @@
     </row>
     <row r="66" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A66" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B66" s="8" t="s">
         <v>5</v>
@@ -47511,7 +47511,7 @@
     </row>
     <row r="67" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A67" s="12" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>4</v>
@@ -47939,7 +47939,7 @@
     </row>
     <row r="71" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A71" s="4" t="s">
-        <v>51</v>
+        <v>116</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>4</v>
@@ -48046,7 +48046,7 @@
     </row>
     <row r="72" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A72" s="29" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B72" s="30" t="s">
         <v>4</v>
@@ -48153,7 +48153,7 @@
     </row>
     <row r="73" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A73" s="29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B73" s="30" t="s">
         <v>4</v>
@@ -48367,7 +48367,7 @@
     </row>
     <row r="75" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A75" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B75" s="4" t="s">
         <v>4</v>
@@ -48474,7 +48474,7 @@
     </row>
     <row r="76" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A76" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B76" s="4" t="s">
         <v>4</v>
@@ -48581,7 +48581,7 @@
     </row>
     <row r="77" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A77" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B77" s="4" t="s">
         <v>4</v>
@@ -48688,7 +48688,7 @@
     </row>
     <row r="78" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A78" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B78" s="4" t="s">
         <v>4</v>
@@ -48795,7 +48795,7 @@
     </row>
     <row r="79" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A79" s="12" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B79" s="4" t="s">
         <v>4</v>
@@ -48902,7 +48902,7 @@
     </row>
     <row r="80" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A80" s="29" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B80" s="30" t="s">
         <v>4</v>
@@ -49009,7 +49009,7 @@
     </row>
     <row r="81" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A81" s="29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B81" s="30" t="s">
         <v>4</v>
@@ -49116,7 +49116,7 @@
     </row>
     <row r="82" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A82" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B82" s="4" t="s">
         <v>4</v>
@@ -49223,7 +49223,7 @@
     </row>
     <row r="83" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A83" s="12" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B83" s="4" t="s">
         <v>4</v>
@@ -49330,7 +49330,7 @@
     </row>
     <row r="84" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A84" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B84" s="4" t="s">
         <v>4</v>
@@ -49437,7 +49437,7 @@
     </row>
     <row r="85" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A85" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B85" s="8" t="s">
         <v>5</v>
@@ -49544,7 +49544,7 @@
     </row>
     <row r="86" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A86" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B86" s="4" t="s">
         <v>4</v>
@@ -49651,7 +49651,7 @@
     </row>
     <row r="87" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A87" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>11</v>
@@ -49758,7 +49758,7 @@
     </row>
     <row r="88" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A88" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B88" s="4" t="s">
         <v>4</v>
@@ -49865,7 +49865,7 @@
     </row>
     <row r="89" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A89" s="12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>4</v>
@@ -49972,7 +49972,7 @@
     </row>
     <row r="90" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A90" s="12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B90" s="4" t="s">
         <v>4</v>
@@ -50079,7 +50079,7 @@
     </row>
     <row r="91" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A91" s="12" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B91" s="4" t="s">
         <v>4</v>
@@ -50186,7 +50186,7 @@
     </row>
     <row r="92" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A92" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B92" s="4" t="s">
         <v>4</v>
@@ -50293,7 +50293,7 @@
     </row>
     <row r="93" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A93" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B93" s="8" t="s">
         <v>5</v>
@@ -50400,7 +50400,7 @@
     </row>
     <row r="94" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A94" s="12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B94" s="4" t="s">
         <v>4</v>
@@ -50507,7 +50507,7 @@
     </row>
     <row r="95" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A95" s="12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B95" s="4" t="s">
         <v>4</v>
@@ -50614,7 +50614,7 @@
     </row>
     <row r="96" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A96" s="12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B96" s="4" t="s">
         <v>4</v>
@@ -50721,7 +50721,7 @@
     </row>
     <row r="97" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A97" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B97" s="4" t="s">
         <v>4</v>
@@ -50828,7 +50828,7 @@
     </row>
     <row r="98" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A98" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B98" s="4" t="s">
         <v>4</v>
@@ -50935,7 +50935,7 @@
     </row>
     <row r="99" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A99" s="28" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B99" s="28" t="s">
         <v>4</v>
@@ -51042,13 +51042,13 @@
     </row>
     <row r="100" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A100" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B100" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D100" s="2">
         <v>0</v>
@@ -51149,13 +51149,13 @@
     </row>
     <row r="101" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A101" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B101" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D101" s="2">
         <v>0</v>
@@ -51256,13 +51256,13 @@
     </row>
     <row r="102" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A102" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C102" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="B102" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C102" s="1" t="s">
-        <v>80</v>
       </c>
       <c r="D102" s="2">
         <v>0</v>
@@ -51363,7 +51363,7 @@
     </row>
     <row r="103" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A103" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B103" s="8" t="s">
         <v>5</v>
@@ -51470,7 +51470,7 @@
     </row>
     <row r="104" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A104" s="28" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B104" s="28" t="s">
         <v>4</v>
@@ -51577,7 +51577,7 @@
     </row>
     <row r="105" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A105" s="12" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B105" s="4" t="s">
         <v>4</v>
@@ -51684,7 +51684,7 @@
     </row>
     <row r="106" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A106" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B106" s="4" t="s">
         <v>4</v>
@@ -51791,7 +51791,7 @@
     </row>
     <row r="107" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A107" s="12" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B107" s="4" t="s">
         <v>4</v>
@@ -51898,7 +51898,7 @@
     </row>
     <row r="108" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A108" s="28" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B108" s="28" t="s">
         <v>4</v>
@@ -52005,7 +52005,7 @@
     </row>
     <row r="109" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A109" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B109" s="8" t="s">
         <v>5</v>
@@ -52112,10 +52112,10 @@
     </row>
     <row r="110" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A110" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B110" s="4" t="s">
         <v>85</v>
-      </c>
-      <c r="B110" s="4" t="s">
-        <v>86</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>8</v>
@@ -52219,10 +52219,10 @@
     </row>
     <row r="111" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A111" s="28" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B111" s="28" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>2</v>
@@ -52326,10 +52326,10 @@
     </row>
     <row r="112" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A112" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B112" s="12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>2</v>
@@ -52340,106 +52340,106 @@
       <c r="E112" s="2">
         <v>0</v>
       </c>
-      <c r="F112" s="2">
-        <v>0</v>
-      </c>
-      <c r="G112" s="2">
-        <v>0</v>
-      </c>
-      <c r="H112" s="2">
-        <v>0</v>
-      </c>
-      <c r="I112" s="2">
-        <v>0</v>
-      </c>
-      <c r="J112" s="2">
-        <v>0</v>
-      </c>
-      <c r="K112" s="2">
-        <v>0</v>
-      </c>
-      <c r="L112" s="2">
-        <v>0</v>
-      </c>
-      <c r="M112" s="2">
-        <v>0</v>
-      </c>
-      <c r="N112" s="2">
-        <v>0</v>
-      </c>
-      <c r="O112" s="2">
-        <v>0</v>
-      </c>
-      <c r="P112" s="2">
-        <v>0</v>
-      </c>
-      <c r="Q112" s="2">
-        <v>0</v>
-      </c>
-      <c r="R112" s="2">
-        <v>0</v>
-      </c>
-      <c r="S112" s="2">
-        <v>0</v>
-      </c>
-      <c r="T112" s="2">
-        <v>0</v>
-      </c>
-      <c r="U112" s="2">
-        <v>0</v>
-      </c>
-      <c r="V112" s="2">
-        <v>0</v>
-      </c>
-      <c r="W112" s="2">
-        <v>0</v>
-      </c>
-      <c r="X112" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y112" s="2">
-        <v>0</v>
-      </c>
-      <c r="Z112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AD112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AE112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AF112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AG112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AH112" s="2">
-        <v>0</v>
-      </c>
-      <c r="AI112" s="2">
-        <v>0</v>
+      <c r="F112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="G112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="H112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="I112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="J112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="K112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="L112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="M112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="N112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="O112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="P112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="R112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="S112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="T112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="U112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="V112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="W112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="X112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="Y112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="Z112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AA112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AB112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AC112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AD112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AE112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AF112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AG112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AH112" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="AI112" s="27" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="113" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A113" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B113" s="12" t="s">
         <v>89</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D113" s="2">
         <v>0</v>
@@ -52540,13 +52540,13 @@
     </row>
     <row r="114" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A114" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B114" s="12" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D114" s="2">
         <v>0</v>
@@ -52647,10 +52647,10 @@
     </row>
     <row r="115" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A115" s="28" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B115" s="28" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>2</v>
@@ -52754,10 +52754,10 @@
     </row>
     <row r="116" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A116" s="28" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B116" s="28" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>2</v>
@@ -52861,10 +52861,10 @@
     </row>
     <row r="117" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A117" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B117" s="12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>2</v>
@@ -52968,10 +52968,10 @@
     </row>
     <row r="118" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A118" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B118" s="12" t="s">
         <v>92</v>
-      </c>
-      <c r="B118" s="12" t="s">
-        <v>93</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>2</v>
@@ -53075,10 +53075,10 @@
     </row>
     <row r="119" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A119" s="28" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B119" s="28" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>2</v>
@@ -53182,10 +53182,10 @@
     </row>
     <row r="120" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A120" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C120" s="1" t="s">
         <v>8</v>
@@ -53289,10 +53289,10 @@
     </row>
     <row r="121" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A121" s="28" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B121" s="28" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C121" s="1" t="s">
         <v>2</v>

</xml_diff>